<commit_message>
data: final SFO addition — MacAndrews & Forbes (Perelman); batch 3 closes the expansion
Final pre-deadline batch: 15 candidates (eight retries with a new direct-fetch fallback
for sites Firecrawl could not read, seven newly researched). One passed the gate:
MacAndrews & Forbes Incorporated - "Wholly owned by Chairman and Chief Executive Officer
Ronald O. Perelman" - the single-owner investment-holding class of the accepted KIRKBI
and Artemis records. Fourteen rejected on the record, eight because their sites could
not be read even with the direct-fetch fallback: the measured edge of the free-tier
verifiable universe, now documented in D26.

Delivered set 60 -> 61; SFO 9 -> 10. Docs reconciled; suite 97 passed; eval 29/29.
</commit_message>
<xml_diff>
--- a/data/final/family_offices.xlsx
+++ b/data/final/family_offices.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT61"/>
+  <dimension ref="A1:AT62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8948,6 +8948,122 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>fo_e6bc01c928</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>MacAndrews &amp; Forbes Incorporated</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Single-Family Office</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Firm's own website self-identifies as a single-owner investment holding: "Wholly owned by Chairman and Chief Executive Officer Ronald O. Perelman" — the diversified investment holding of one named individual, the same class as the accepted KIRKBI and Artémis records. Discovered via a curated-reference lens; verified against the firm's own website.</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Diversified investment holding company wholly owned by Ronald O. Perelman.</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Our core strategy is to focus our business lines on strong market positions, high quality management with vertical expertise, recognized growth potential and ability to increase profitability.</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>https://www.macandrewsandforbes.com/</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr"/>
+      <c r="T62" t="inlineStr"/>
+      <c r="U62" t="inlineStr"/>
+      <c r="V62" t="inlineStr"/>
+      <c r="W62" t="inlineStr"/>
+      <c r="X62" t="inlineStr"/>
+      <c r="Y62" t="inlineStr"/>
+      <c r="Z62" t="inlineStr"/>
+      <c r="AA62" t="inlineStr"/>
+      <c r="AB62" t="inlineStr"/>
+      <c r="AC62" t="inlineStr"/>
+      <c r="AD62" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AE62" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AF62" t="inlineStr"/>
+      <c r="AG62" t="inlineStr"/>
+      <c r="AH62" t="inlineStr"/>
+      <c r="AI62" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AJ62" t="inlineStr"/>
+      <c r="AK62" t="inlineStr"/>
+      <c r="AL62" t="inlineStr"/>
+      <c r="AM62" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AN62" t="inlineStr"/>
+      <c r="AO62" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="AP62" t="inlineStr">
+        <is>
+          <t>Firm Website (single-family-office status, firm identity)</t>
+        </is>
+      </c>
+      <c r="AQ62" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AR62" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="AS62" t="inlineStr">
+        <is>
+          <t>estimated_aum; corporate_linkedin; principal_name; principal_title; principal_linkedin; principal_email; principal_phone; hq_phone</t>
+        </is>
+      </c>
+      <c r="AT62" t="inlineStr">
+        <is>
+          <t>Discovered via the curated/notable-reference lens; classification and firm identity verified against the firm's own authoritative website (single verification source). AUM and individual contact details are not available from free authoritative sources and are left could_not_verify. Perelman is the owner; the site names no separate office decision-maker, so principal fields stay blank. Geography is not stated on the scraped pages and is left blank.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8959,7 +9075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H414"/>
+  <dimension ref="A1:H419"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25153,6 +25269,196 @@
         </is>
       </c>
       <c r="H414" t="inlineStr"/>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>fo_e6bc01c928</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>https://www.macandrewsandforbes.com/</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr"/>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>fo_e6bc01c928</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>https://www.macandrewsandforbes.com/</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr"/>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>fo_e6bc01c928</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>https://www.macandrewsandforbes.com/</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr"/>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>fo_e6bc01c928</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>investment_thesis</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>https://www.macandrewsandforbes.com/</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr"/>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>fo_e6bc01c928</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>fo_type_evidence</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>https://www.macandrewsandforbes.com/</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25165,7 +25471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F166"/>
+  <dimension ref="A1:F168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29995,6 +30301,62 @@
       <c r="D166" t="inlineStr"/>
       <c r="E166" t="inlineStr"/>
       <c r="F166" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>fo_e6bc01c928</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>verification</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>single-family-office status, firm identity</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>https://www.macandrewsandforbes.com/</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>fo_e6bc01c928</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr"/>
+      <c r="E168" t="inlineStr"/>
+      <c r="F168" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>

</xml_diff>

<commit_message>
chore(data): autonomous data update via operating cycle
</commit_message>
<xml_diff>
--- a/data/final/family_offices.xlsx
+++ b/data/final/family_offices.xlsx
@@ -2139,12 +2139,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>fo_9220a272d8</t>
+          <t>fo_15eb1b42d3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Custos Family Office, LLC</t>
+          <t>Tarbox Family Office, Inc.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2154,31 +2154,23 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>SEC 13F filer self-identifying as a family office; SEC Form ADV / IAPD registration names it a family office; firm website describes itself as a family office; type: single vs multi family not established</t>
+          <t>SEC 13F filer self-identifying as a family office; SEC Form ADV / IAPD registration names it a family office; type: single vs multi family not established</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>We function as our clients’ Chief Financial Officer – protecting their wealth, coordinating financial services through the families’ various stages, and acting as a bridge across generations.</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>https://custosfo.com/</t>
-        </is>
-      </c>
+      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>AUSTIN</t>
+          <t>NEWPORT BEACH</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -2188,7 +2180,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>+1 (303) 578-7024</t>
+          <t>+1 (949) 721-2330</t>
         </is>
       </c>
       <c r="O14" t="inlineStr"/>
@@ -2219,19 +2211,11 @@
       <c r="AF14" t="inlineStr"/>
       <c r="AG14" t="inlineStr"/>
       <c r="AH14" t="inlineStr"/>
-      <c r="AI14" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="AI14" t="inlineStr"/>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
       <c r="AL14" t="inlineStr"/>
-      <c r="AM14" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
+      <c r="AM14" t="inlineStr"/>
       <c r="AN14" t="inlineStr"/>
       <c r="AO14" t="inlineStr">
         <is>
@@ -2240,7 +2224,7 @@
       </c>
       <c r="AP14" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings) (firm existence, address, phone, EIN); SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type); Firm Website (family-office status, type)</t>
+          <t>SEC EDGAR (13F / SC / Form D filings) (firm existence, address, phone, EIN); SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type)</t>
         </is>
       </c>
       <c r="AQ14" t="inlineStr">
@@ -2395,12 +2379,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>fo_15eb1b42d3</t>
+          <t>fo_4b474eef93</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Tarbox Family Office, Inc.</t>
+          <t>Duquesne Family Office LLC</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2421,12 +2405,12 @@
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>NEWPORT BEACH</t>
+          <t>NEW YORK</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2436,7 +2420,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>+1 (949) 721-2330</t>
+          <t>+1 (212) 830-6500</t>
         </is>
       </c>
       <c r="O16" t="inlineStr"/>
@@ -2635,12 +2619,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>fo_4b474eef93</t>
+          <t>fo_3eb2ccad75</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Duquesne Family Office LLC</t>
+          <t>CVA Family Office, LLC</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2661,12 +2645,12 @@
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>NEW YORK</t>
+          <t>DENVER</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2676,7 +2660,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>+1 (212) 830-6500</t>
+          <t>+1 (303) 243-5611</t>
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
@@ -2895,12 +2879,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>fo_3eb2ccad75</t>
+          <t>fo_9220a272d8</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CVA Family Office, LLC</t>
+          <t>Custos Family Office, LLC</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2910,23 +2894,31 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>SEC 13F filer self-identifying as a family office; SEC Form ADV / IAPD registration names it a family office; type: single vs multi family not established</t>
+          <t>SEC 13F filer self-identifying as a family office; SEC Form ADV / IAPD registration names it a family office; firm website describes itself as a family office; type: single vs multi family not established</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>We function as our clients’ Chief Financial Officer – protecting their wealth, coordinating financial services through the families’ various stages, and acting as a bridge across generations.</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://custosfo.com/</t>
+        </is>
+      </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>DENVER</t>
+          <t>AUSTIN</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2936,7 +2928,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>+1 (303) 243-5611</t>
+          <t>+1 (303) 578-7024</t>
         </is>
       </c>
       <c r="O20" t="inlineStr"/>
@@ -2967,11 +2959,19 @@
       <c r="AF20" t="inlineStr"/>
       <c r="AG20" t="inlineStr"/>
       <c r="AH20" t="inlineStr"/>
-      <c r="AI20" t="inlineStr"/>
+      <c r="AI20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
       <c r="AL20" t="inlineStr"/>
-      <c r="AM20" t="inlineStr"/>
+      <c r="AM20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
       <c r="AN20" t="inlineStr"/>
       <c r="AO20" t="inlineStr">
         <is>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="AP20" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings) (firm existence, address, phone, EIN); SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type)</t>
+          <t>SEC EDGAR (13F / SC / Form D filings) (firm existence, address, phone, EIN); SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type); Firm Website (family-office status, type)</t>
         </is>
       </c>
       <c r="AQ20" t="inlineStr">
@@ -3635,12 +3635,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>fo_89137929e9</t>
+          <t>fo_685bea3a32</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BOSTON FAMILY OFFICE LLC</t>
+          <t>Kopp Family Office, LLC</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3661,12 +3661,12 @@
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>BOSTON</t>
+          <t>MINNETONKA</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3676,7 +3676,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>+1 (617) 624-0800</t>
+          <t>+1 (952) 841-0400</t>
         </is>
       </c>
       <c r="O26" t="inlineStr"/>
@@ -3875,12 +3875,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>fo_da95e70bda</t>
+          <t>fo_89137929e9</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Fortitude Family Office, LLC</t>
+          <t>BOSTON FAMILY OFFICE LLC</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3890,31 +3890,23 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>SEC 13F filer self-identifying as a family office; SEC Form ADV / IAPD registration names it a family office; firm website describes itself as a family office; type: single vs multi family not established</t>
+          <t>SEC 13F filer self-identifying as a family office; SEC Form ADV / IAPD registration names it a family office; type: single vs multi family not established</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Investments Our in-house investment team will craft custom, goals-based, and integrated strategies to not just keep your wealth, but grow it.</t>
-        </is>
-      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>https://fortitudefo.com/</t>
-        </is>
-      </c>
+      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>SCOTTSDALE</t>
+          <t>BOSTON</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3924,7 +3916,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>+1 (602) 834-0089</t>
+          <t>+1 (617) 624-0800</t>
         </is>
       </c>
       <c r="O28" t="inlineStr"/>
@@ -3955,19 +3947,11 @@
       <c r="AF28" t="inlineStr"/>
       <c r="AG28" t="inlineStr"/>
       <c r="AH28" t="inlineStr"/>
-      <c r="AI28" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="AI28" t="inlineStr"/>
       <c r="AJ28" t="inlineStr"/>
       <c r="AK28" t="inlineStr"/>
       <c r="AL28" t="inlineStr"/>
-      <c r="AM28" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
+      <c r="AM28" t="inlineStr"/>
       <c r="AN28" t="inlineStr"/>
       <c r="AO28" t="inlineStr">
         <is>
@@ -3976,7 +3960,7 @@
       </c>
       <c r="AP28" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings) (firm existence, address, phone, EIN); SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type); Firm Website (family-office status, type)</t>
+          <t>SEC EDGAR (13F / SC / Form D filings) (firm existence, address, phone, EIN); SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type)</t>
         </is>
       </c>
       <c r="AQ28" t="inlineStr">
@@ -4144,12 +4128,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>fo_29e17a89bc</t>
+          <t>fo_da95e70bda</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Pioneer Family Office, LLC</t>
+          <t>Fortitude Family Office, LLC</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -4159,23 +4143,31 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>SEC 13F filer self-identifying as a family office; SEC Form ADV / IAPD registration names it a family office; type: single vs multi family not established</t>
+          <t>SEC 13F filer self-identifying as a family office; SEC Form ADV / IAPD registration names it a family office; firm website describes itself as a family office; type: single vs multi family not established</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Investments Our in-house investment team will craft custom, goals-based, and integrated strategies to not just keep your wealth, but grow it.</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>https://fortitudefo.com/</t>
+        </is>
+      </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>NORTH MIAMI BEACH</t>
+          <t>SCOTTSDALE</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -4185,7 +4177,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>+1 (305) 935-5502</t>
+          <t>+1 (602) 834-0089</t>
         </is>
       </c>
       <c r="O30" t="inlineStr"/>
@@ -4216,11 +4208,19 @@
       <c r="AF30" t="inlineStr"/>
       <c r="AG30" t="inlineStr"/>
       <c r="AH30" t="inlineStr"/>
-      <c r="AI30" t="inlineStr"/>
+      <c r="AI30" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
       <c r="AJ30" t="inlineStr"/>
       <c r="AK30" t="inlineStr"/>
       <c r="AL30" t="inlineStr"/>
-      <c r="AM30" t="inlineStr"/>
+      <c r="AM30" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
       <c r="AN30" t="inlineStr"/>
       <c r="AO30" t="inlineStr">
         <is>
@@ -4229,7 +4229,7 @@
       </c>
       <c r="AP30" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings) (firm existence, address, phone, EIN); SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type)</t>
+          <t>SEC EDGAR (13F / SC / Form D filings) (firm existence, address, phone, EIN); SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type); Firm Website (family-office status, type)</t>
         </is>
       </c>
       <c r="AQ30" t="inlineStr">
@@ -4384,12 +4384,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>fo_685bea3a32</t>
+          <t>fo_beb7590905</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Kopp Family Office, LLC</t>
+          <t>Callan Family Office, LLC</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -4399,23 +4399,35 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>SEC 13F filer self-identifying as a family office; SEC Form ADV / IAPD registration names it a family office; type: single vs multi family not established</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
+          <t>SEC 13F filer self-identifying as a family office; SEC Form ADV / IAPD registration names it a family office; firm website describes itself as a family office; type: single vs multi family not established</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>A partnership of entrepreneurs serving entrepreneurial families, Callan Family Office’s 23 partners have decades of experience working exclusively with ultra-high-net-worth families across generations. We operate as an independent firm, offering tailored, open-architecture solutions that integrate seamlessly into every aspect of your financial life. As a fiduciary, we are committed to prioritizing</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Get Started Tax-Focused Planning and Investments For ultra-high-net-worth families, tax-efficient investment and planning are paramount to growing and preserving wealth across generations.</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>https://callanfamilyoffice.com/</t>
+        </is>
+      </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
-          <t>MINNETONKA</t>
+          <t>RADNOR</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -4425,7 +4437,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>+1 (952) 841-0400</t>
+          <t>+1 (267) 250-2036</t>
         </is>
       </c>
       <c r="O32" t="inlineStr"/>
@@ -4456,11 +4468,19 @@
       <c r="AF32" t="inlineStr"/>
       <c r="AG32" t="inlineStr"/>
       <c r="AH32" t="inlineStr"/>
-      <c r="AI32" t="inlineStr"/>
+      <c r="AI32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
       <c r="AJ32" t="inlineStr"/>
       <c r="AK32" t="inlineStr"/>
       <c r="AL32" t="inlineStr"/>
-      <c r="AM32" t="inlineStr"/>
+      <c r="AM32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
       <c r="AN32" t="inlineStr"/>
       <c r="AO32" t="inlineStr">
         <is>
@@ -4469,7 +4489,7 @@
       </c>
       <c r="AP32" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings) (firm existence, address, phone, EIN); SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type)</t>
+          <t>SEC EDGAR (13F / SC / Form D filings) (firm existence, address, phone, EIN); SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type); Firm Website (family-office status, type)</t>
         </is>
       </c>
       <c r="AQ32" t="inlineStr">
@@ -4624,12 +4644,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>fo_beb7590905</t>
+          <t>fo_29e17a89bc</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Callan Family Office, LLC</t>
+          <t>Pioneer Family Office, LLC</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -4639,35 +4659,23 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>SEC 13F filer self-identifying as a family office; SEC Form ADV / IAPD registration names it a family office; firm website describes itself as a family office; type: single vs multi family not established</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>A partnership of entrepreneurs serving entrepreneurial families, Callan Family Office’s 23 partners have decades of experience working exclusively with ultra-high-net-worth families across generations. We operate as an independent firm, offering tailored, open-architecture solutions that integrate seamlessly into every aspect of your financial life. As a fiduciary, we are committed to prioritizing</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Get Started Tax-Focused Planning and Investments For ultra-high-net-worth families, tax-efficient investment and planning are paramount to growing and preserving wealth across generations.</t>
-        </is>
-      </c>
+          <t>SEC 13F filer self-identifying as a family office; SEC Form ADV / IAPD registration names it a family office; type: single vs multi family not established</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>https://callanfamilyoffice.com/</t>
-        </is>
-      </c>
+      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>RADNOR</t>
+          <t>NORTH MIAMI BEACH</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4677,7 +4685,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>+1 (267) 250-2036</t>
+          <t>+1 (305) 935-5502</t>
         </is>
       </c>
       <c r="O34" t="inlineStr"/>
@@ -4708,19 +4716,11 @@
       <c r="AF34" t="inlineStr"/>
       <c r="AG34" t="inlineStr"/>
       <c r="AH34" t="inlineStr"/>
-      <c r="AI34" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="AI34" t="inlineStr"/>
       <c r="AJ34" t="inlineStr"/>
       <c r="AK34" t="inlineStr"/>
       <c r="AL34" t="inlineStr"/>
-      <c r="AM34" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
+      <c r="AM34" t="inlineStr"/>
       <c r="AN34" t="inlineStr"/>
       <c r="AO34" t="inlineStr">
         <is>
@@ -4729,7 +4729,7 @@
       </c>
       <c r="AP34" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings) (firm existence, address, phone, EIN); SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type); Firm Website (family-office status, type)</t>
+          <t>SEC EDGAR (13F / SC / Form D filings) (firm existence, address, phone, EIN); SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type)</t>
         </is>
       </c>
       <c r="AQ34" t="inlineStr">
@@ -11345,7 +11345,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>fo_9220a272d8</t>
+          <t>fo_15eb1b42d3</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -11365,7 +11365,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001904423.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001599603.json</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -11383,7 +11383,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>fo_9220a272d8</t>
+          <t>fo_15eb1b42d3</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001904423.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001599603.json</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -11421,7 +11421,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>fo_9220a272d8</t>
+          <t>fo_15eb1b42d3</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -11441,7 +11441,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001904423.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001599603.json</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -11459,12 +11459,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>fo_9220a272d8</t>
+          <t>fo_a4cb68cd35</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>website</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -11474,17 +11474,17 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>fetched firm website</t>
+          <t>firm website</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>https://custosfo.com/</t>
+          <t>https://matterfamilyoffice.com</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -11497,32 +11497,32 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>fo_9220a272d8</t>
+          <t>fo_a4cb68cd35</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>investment_thesis</t>
+          <t>hq_country</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>firm website (stated investment approach / mission)</t>
+          <t>IAPD registration record</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>https://custosfo.com/</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/106806</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -11540,7 +11540,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>website</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -11550,17 +11550,17 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>firm website</t>
+          <t>fetched firm website</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>https://matterfamilyoffice.com</t>
+          <t>https://www.matterfamilyoffice.com/</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -11578,27 +11578,27 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>hq_country</t>
+          <t>description</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>IAPD registration record</t>
+          <t>website meta description</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/106806</t>
+          <t>https://www.matterfamilyoffice.com/</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -11616,7 +11616,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>website</t>
+          <t>investment_thesis</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -11626,7 +11626,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>fetched firm website</t>
+          <t>firm website (stated investment approach / mission)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -11636,7 +11636,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -11649,32 +11649,32 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>fo_a4cb68cd35</t>
+          <t>fo_4b474eef93</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>website meta description</t>
+          <t>SEC EDGAR submissions (registrant name)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>https://www.matterfamilyoffice.com/</t>
+          <t>https://data.sec.gov/submissions/CIK0001536411.json</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -11687,32 +11687,32 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>fo_a4cb68cd35</t>
+          <t>fo_4b474eef93</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>investment_thesis</t>
+          <t>hq_country</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>firm website (stated investment approach / mission)</t>
+          <t>SEC EDGAR submissions (business address)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>https://www.matterfamilyoffice.com/</t>
+          <t>https://data.sec.gov/submissions/CIK0001536411.json</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -11725,12 +11725,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>fo_15eb1b42d3</t>
+          <t>fo_4b474eef93</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>hq_phone</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -11740,12 +11740,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>SEC EDGAR submissions (registrant name)</t>
+          <t>SEC EDGAR submissions (business phone)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001599603.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001536411.json</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -11763,32 +11763,32 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>fo_15eb1b42d3</t>
+          <t>fo_55e904bc2b</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>hq_country</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>SEC EDGAR submissions (business address)</t>
+          <t>firm website</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001599603.json</t>
+          <t>https://sestantefo.com</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -11801,27 +11801,27 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>fo_15eb1b42d3</t>
+          <t>fo_55e904bc2b</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>hq_phone</t>
+          <t>hq_country</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>SEC EDGAR submissions (business phone)</t>
+          <t>IAPD registration record</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001599603.json</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/335152</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -11844,7 +11844,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>website</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -11854,17 +11854,17 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>firm website</t>
+          <t>fetched firm website</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>https://sestantefamilyoffice.com</t>
+          <t>http://sestante.com/</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -11882,27 +11882,27 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>hq_country</t>
+          <t>description</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>IAPD registration record</t>
+          <t>website meta description</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/335152</t>
+          <t>http://sestante.com/</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -11920,7 +11920,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>website</t>
+          <t>investment_thesis</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -11930,7 +11930,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>fetched firm website</t>
+          <t>firm website (stated investment approach / mission)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -11940,7 +11940,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -11953,32 +11953,32 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>fo_55e904bc2b</t>
+          <t>fo_3eb2ccad75</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>website meta description</t>
+          <t>SEC EDGAR submissions (registrant name)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>http://sestante.com/</t>
+          <t>https://data.sec.gov/submissions/CIK0001802084.json</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -11991,32 +11991,32 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>fo_55e904bc2b</t>
+          <t>fo_3eb2ccad75</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>investment_thesis</t>
+          <t>hq_country</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>firm website (stated investment approach / mission)</t>
+          <t>SEC EDGAR submissions (business address)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>http://sestante.com/</t>
+          <t>https://data.sec.gov/submissions/CIK0001802084.json</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -12029,12 +12029,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>fo_4b474eef93</t>
+          <t>fo_3eb2ccad75</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>hq_phone</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -12044,12 +12044,12 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>SEC EDGAR submissions (registrant name)</t>
+          <t>SEC EDGAR submissions (business phone)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001536411.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001802084.json</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -12067,32 +12067,32 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>fo_4b474eef93</t>
+          <t>fo_f638fbd06f</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>hq_country</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>SEC EDGAR submissions (business address)</t>
+          <t>firm website</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001536411.json</t>
+          <t>https://storyonefamilyoffice.com</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -12105,27 +12105,27 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>fo_4b474eef93</t>
+          <t>fo_f638fbd06f</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>hq_phone</t>
+          <t>hq_country</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>SEC EDGAR submissions (business phone)</t>
+          <t>IAPD registration record</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001536411.json</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/331394</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -12148,7 +12148,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>website</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -12158,17 +12158,17 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>firm website</t>
+          <t>fetched firm website</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>https://storyonefamilyoffice.com</t>
+          <t>https://story-one.com/</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -12186,27 +12186,27 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>hq_country</t>
+          <t>description</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>IAPD registration record</t>
+          <t>website meta description</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/331394</t>
+          <t>https://story-one.com/</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -12224,7 +12224,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>website</t>
+          <t>investment_thesis</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -12234,7 +12234,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>fetched firm website</t>
+          <t>firm website (stated investment approach / mission)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -12244,7 +12244,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -12262,27 +12262,27 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>estimated_aum</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>website meta description</t>
+          <t>SEC Form ADV Part 1A (Item 5.F total AUM / Schedule A control person)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>https://story-one.com/</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/331394</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -12300,27 +12300,27 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>investment_thesis</t>
+          <t>principal_name</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>firm website (stated investment approach / mission)</t>
+          <t>SEC Form ADV Part 1A (Item 5.F total AUM / Schedule A control person)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>https://story-one.com/</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/331394</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -12338,7 +12338,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>estimated_aum</t>
+          <t>principal_title</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -12371,27 +12371,27 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>fo_f638fbd06f</t>
+          <t>fo_9220a272d8</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>principal_name</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>SEC Form ADV Part 1A (Item 5.F total AUM / Schedule A control person)</t>
+          <t>SEC EDGAR submissions (registrant name)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/331394</t>
+          <t>https://data.sec.gov/submissions/CIK0001904423.json</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -12409,27 +12409,27 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>fo_f638fbd06f</t>
+          <t>fo_9220a272d8</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>principal_title</t>
+          <t>hq_country</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>SEC Form ADV Part 1A (Item 5.F total AUM / Schedule A control person)</t>
+          <t>SEC EDGAR submissions (business address)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/331394</t>
+          <t>https://data.sec.gov/submissions/CIK0001904423.json</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -12447,12 +12447,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>fo_3eb2ccad75</t>
+          <t>fo_9220a272d8</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>hq_phone</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -12462,12 +12462,12 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>SEC EDGAR submissions (registrant name)</t>
+          <t>SEC EDGAR submissions (business phone)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001802084.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001904423.json</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -12485,27 +12485,27 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>fo_3eb2ccad75</t>
+          <t>fo_9220a272d8</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>hq_country</t>
+          <t>website</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>SEC EDGAR submissions (business address)</t>
+          <t>fetched firm website</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001802084.json</t>
+          <t>https://custosfo.com/</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -12523,32 +12523,32 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>fo_3eb2ccad75</t>
+          <t>fo_9220a272d8</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>hq_phone</t>
+          <t>investment_thesis</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>SEC EDGAR submissions (business phone)</t>
+          <t>firm website (stated investment approach / mission)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001802084.json</t>
+          <t>https://custosfo.com/</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -13473,7 +13473,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>fo_89137929e9</t>
+          <t>fo_685bea3a32</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -13493,7 +13493,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001039807.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001683689.json</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13511,7 +13511,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>fo_89137929e9</t>
+          <t>fo_685bea3a32</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -13531,7 +13531,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001039807.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001683689.json</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13549,7 +13549,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>fo_89137929e9</t>
+          <t>fo_685bea3a32</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -13569,7 +13569,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001039807.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001683689.json</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -13777,7 +13777,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>fo_da95e70bda</t>
+          <t>fo_89137929e9</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -13797,7 +13797,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001950506.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001039807.json</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -13815,7 +13815,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>fo_da95e70bda</t>
+          <t>fo_89137929e9</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -13835,7 +13835,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001950506.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001039807.json</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -13853,7 +13853,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>fo_da95e70bda</t>
+          <t>fo_89137929e9</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -13873,7 +13873,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001950506.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001039807.json</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -13891,12 +13891,12 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>fo_da95e70bda</t>
+          <t>fo_80f649ced1</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>website</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -13906,17 +13906,17 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>fetched firm website</t>
+          <t>firm website</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>https://fortitudefo.com/</t>
+          <t>https://dcafamilyoffice.com</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -13929,32 +13929,32 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>fo_da95e70bda</t>
+          <t>fo_80f649ced1</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>investment_thesis</t>
+          <t>hq_country</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>firm website (stated investment approach / mission)</t>
+          <t>IAPD registration record</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>https://fortitudefo.com/</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/322047</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -13972,7 +13972,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>website</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -13982,17 +13982,17 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>firm website</t>
+          <t>fetched firm website</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>https://dcafamilyoffice.com</t>
+          <t>https://dcafamilyoffice.com/</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -14010,27 +14010,27 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>hq_country</t>
+          <t>description</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>IAPD registration record</t>
+          <t>website meta description</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/322047</t>
+          <t>https://dcafamilyoffice.com/</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -14048,22 +14048,22 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>website</t>
+          <t>estimated_aum</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>fetched firm website</t>
+          <t>SEC Form ADV Part 1A (Item 5.F total AUM / Schedule A control person)</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>https://dcafamilyoffice.com/</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/322047</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -14086,27 +14086,27 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>principal_name</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>website meta description</t>
+          <t>SEC Form ADV Part 1A (Item 5.F total AUM / Schedule A control person)</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>https://dcafamilyoffice.com/</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/322047</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
@@ -14124,7 +14124,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>estimated_aum</t>
+          <t>principal_title</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -14157,27 +14157,27 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>fo_80f649ced1</t>
+          <t>fo_da95e70bda</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>principal_name</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>SEC Form ADV Part 1A (Item 5.F total AUM / Schedule A control person)</t>
+          <t>SEC EDGAR submissions (registrant name)</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/322047</t>
+          <t>https://data.sec.gov/submissions/CIK0001950506.json</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -14195,27 +14195,27 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>fo_80f649ced1</t>
+          <t>fo_da95e70bda</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>principal_title</t>
+          <t>hq_country</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>SEC Form ADV Part 1A (Item 5.F total AUM / Schedule A control person)</t>
+          <t>SEC EDGAR submissions (business address)</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/322047</t>
+          <t>https://data.sec.gov/submissions/CIK0001950506.json</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -14233,12 +14233,12 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>fo_29e17a89bc</t>
+          <t>fo_da95e70bda</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>hq_phone</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -14248,12 +14248,12 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>SEC EDGAR submissions (registrant name)</t>
+          <t>SEC EDGAR submissions (business phone)</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0002135110.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001950506.json</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -14271,27 +14271,27 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>fo_29e17a89bc</t>
+          <t>fo_da95e70bda</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>hq_country</t>
+          <t>website</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>SEC EDGAR submissions (business address)</t>
+          <t>fetched firm website</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0002135110.json</t>
+          <t>https://fortitudefo.com/</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -14309,32 +14309,32 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>fo_29e17a89bc</t>
+          <t>fo_da95e70bda</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>hq_phone</t>
+          <t>investment_thesis</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>SEC EDGAR submissions (business phone)</t>
+          <t>firm website (stated investment approach / mission)</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0002135110.json</t>
+          <t>https://fortitudefo.com/</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -14537,7 +14537,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>fo_685bea3a32</t>
+          <t>fo_beb7590905</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -14557,7 +14557,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001683689.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001938970.json</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -14575,7 +14575,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>fo_685bea3a32</t>
+          <t>fo_beb7590905</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -14595,7 +14595,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001683689.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001938970.json</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -14613,7 +14613,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>fo_685bea3a32</t>
+          <t>fo_beb7590905</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -14633,7 +14633,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001683689.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001938970.json</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -14651,12 +14651,12 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>fo_3171716a52</t>
+          <t>fo_beb7590905</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>website</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -14666,17 +14666,17 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>firm website</t>
+          <t>fetched firm website</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>https://angelesfamilyoffice.com</t>
+          <t>https://callanfamilyoffice.com/</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -14689,32 +14689,32 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>fo_3171716a52</t>
+          <t>fo_beb7590905</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>hq_country</t>
+          <t>description</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>IAPD registration record</t>
+          <t>website meta description</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/338266</t>
+          <t>https://callanfamilyoffice.com/</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -14727,12 +14727,12 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>fo_3171716a52</t>
+          <t>fo_beb7590905</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>website</t>
+          <t>investment_thesis</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -14742,17 +14742,17 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>fetched firm website</t>
+          <t>firm website (stated investment approach / mission)</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>https://www.angelesinvestments.com/</t>
+          <t>https://callanfamilyoffice.com/</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -14770,7 +14770,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -14780,12 +14780,12 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>website meta description</t>
+          <t>firm website</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>https://www.angelesinvestments.com/</t>
+          <t>https://angelesfamilyoffice.com</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -14808,27 +14808,27 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>investment_thesis</t>
+          <t>hq_country</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>firm website (stated investment approach / mission)</t>
+          <t>IAPD registration record</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>https://www.angelesinvestments.com/</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/338266</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -14841,27 +14841,27 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>fo_beb7590905</t>
+          <t>fo_3171716a52</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>website</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>SEC EDGAR submissions (registrant name)</t>
+          <t>fetched firm website</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001938970.json</t>
+          <t>https://www.angelesinvestments.com/</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -14879,32 +14879,32 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>fo_beb7590905</t>
+          <t>fo_3171716a52</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>hq_country</t>
+          <t>description</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>SEC EDGAR submissions (business address)</t>
+          <t>website meta description</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001938970.json</t>
+          <t>https://www.angelesinvestments.com/</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -14917,32 +14917,32 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>fo_beb7590905</t>
+          <t>fo_3171716a52</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>hq_phone</t>
+          <t>investment_thesis</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>SEC EDGAR submissions (business phone)</t>
+          <t>firm website (stated investment approach / mission)</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001938970.json</t>
+          <t>https://www.angelesinvestments.com/</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -14955,27 +14955,27 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>fo_beb7590905</t>
+          <t>fo_29e17a89bc</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>website</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>fetched firm website</t>
+          <t>SEC EDGAR submissions (registrant name)</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>https://callanfamilyoffice.com/</t>
+          <t>https://data.sec.gov/submissions/CIK0002135110.json</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -14993,32 +14993,32 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>fo_beb7590905</t>
+          <t>fo_29e17a89bc</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>hq_country</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>website meta description</t>
+          <t>SEC EDGAR submissions (business address)</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>https://callanfamilyoffice.com/</t>
+          <t>https://data.sec.gov/submissions/CIK0002135110.json</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -15031,32 +15031,32 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>fo_beb7590905</t>
+          <t>fo_29e17a89bc</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>investment_thesis</t>
+          <t>hq_phone</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>firm website (stated investment approach / mission)</t>
+          <t>SEC EDGAR submissions (business phone)</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>https://callanfamilyoffice.com/</t>
+          <t>https://data.sec.gov/submissions/CIK0002135110.json</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -21967,7 +21967,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>fo_9220a272d8</t>
+          <t>fo_15eb1b42d3</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -21987,7 +21987,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001904423.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001599603.json</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -21999,7 +21999,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>fo_9220a272d8</t>
+          <t>fo_15eb1b42d3</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -22019,7 +22019,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/294025</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/106079</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -22031,29 +22031,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>fo_9220a272d8</t>
+          <t>fo_15eb1b42d3</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>verification</t>
+          <t>discovery</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Firm Website</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>family-office status, type</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>https://custosfo.com/</t>
-        </is>
-      </c>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -22063,21 +22055,29 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>fo_9220a272d8</t>
+          <t>fo_a4cb68cd35</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>verification</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>firm registration, family-office status, type</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://adviserinfo.sec.gov/firm/summary/106806</t>
+        </is>
+      </c>
       <c r="F44" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -22097,17 +22097,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>firm registration, family-office status, type</t>
+          <t>family-office status, type</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/106806</t>
+          <t>https://www.matterfamilyoffice.com/</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -22124,24 +22124,16 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>verification</t>
+          <t>discovery</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Firm Website</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>family-office status, type</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>https://www.matterfamilyoffice.com/</t>
-        </is>
-      </c>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -22151,21 +22143,29 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>fo_a4cb68cd35</t>
+          <t>fo_4b474eef93</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>verification</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>firm existence, address, phone, EIN</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://data.sec.gov/submissions/CIK0001536411.json</t>
+        </is>
+      </c>
       <c r="F47" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -22175,7 +22175,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>fo_15eb1b42d3</t>
+          <t>fo_4b474eef93</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -22185,17 +22185,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>firm existence, address, phone, EIN</t>
+          <t>firm registration, family-office status, type</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001599603.json</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/326761</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -22207,29 +22207,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>fo_15eb1b42d3</t>
+          <t>fo_4b474eef93</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>verification</t>
+          <t>discovery</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>firm registration, family-office status, type</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/106079</t>
-        </is>
-      </c>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -22239,21 +22231,29 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>fo_15eb1b42d3</t>
+          <t>fo_55e904bc2b</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>verification</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>firm registration, family-office status, type</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://adviserinfo.sec.gov/firm/summary/335152</t>
+        </is>
+      </c>
       <c r="F50" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -22273,17 +22273,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>firm registration, family-office status, type</t>
+          <t>family-office status, type</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/335152</t>
+          <t>http://sestante.com/</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -22300,24 +22300,16 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>verification</t>
+          <t>discovery</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Firm Website</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>family-office status, type</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>http://sestante.com/</t>
-        </is>
-      </c>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -22327,21 +22319,29 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>fo_55e904bc2b</t>
+          <t>fo_3eb2ccad75</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>verification</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>firm existence, address, phone, EIN</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://data.sec.gov/submissions/CIK0001802084.json</t>
+        </is>
+      </c>
       <c r="F53" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -22351,7 +22351,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>fo_4b474eef93</t>
+          <t>fo_3eb2ccad75</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -22361,17 +22361,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>firm existence, address, phone, EIN</t>
+          <t>firm registration, family-office status, type</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001536411.json</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/285035</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -22383,29 +22383,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>fo_4b474eef93</t>
+          <t>fo_3eb2ccad75</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>verification</t>
+          <t>discovery</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>firm registration, family-office status, type</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/326761</t>
-        </is>
-      </c>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -22415,21 +22407,29 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>fo_4b474eef93</t>
+          <t>fo_f638fbd06f</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>verification</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>firm registration, family-office status, type</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://adviserinfo.sec.gov/firm/summary/331394</t>
+        </is>
+      </c>
       <c r="F56" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -22449,17 +22449,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>firm registration, family-office status, type</t>
+          <t>family-office status, type</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/331394</t>
+          <t>https://story-one.com/</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -22481,17 +22481,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>family-office status, type</t>
+          <t>total regulatory AUM (ADV Item 5.F), owner/control person (ADV Schedule A)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://story-one.com/</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/331394</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -22508,7 +22508,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>verification</t>
+          <t>discovery</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -22516,16 +22516,8 @@
           <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>total regulatory AUM (ADV Item 5.F), owner/control person (ADV Schedule A)</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/331394</t>
-        </is>
-      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -22535,21 +22527,29 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>fo_f638fbd06f</t>
+          <t>fo_9220a272d8</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>verification</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>firm existence, address, phone, EIN</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://data.sec.gov/submissions/CIK0001904423.json</t>
+        </is>
+      </c>
       <c r="F60" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -22559,7 +22559,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>fo_3eb2ccad75</t>
+          <t>fo_9220a272d8</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -22569,17 +22569,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>firm existence, address, phone, EIN</t>
+          <t>firm registration, family-office status, type</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001802084.json</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/294025</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -22591,7 +22591,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>fo_3eb2ccad75</t>
+          <t>fo_9220a272d8</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -22601,17 +22601,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>firm registration, family-office status, type</t>
+          <t>family-office status, type</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/285035</t>
+          <t>https://custosfo.com/</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -22623,7 +22623,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>fo_3eb2ccad75</t>
+          <t>fo_9220a272d8</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -23151,7 +23151,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>fo_89137929e9</t>
+          <t>fo_685bea3a32</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -23171,7 +23171,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001039807.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001683689.json</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -23183,7 +23183,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>fo_89137929e9</t>
+          <t>fo_685bea3a32</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -23203,7 +23203,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/107141</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/326761</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -23215,7 +23215,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>fo_89137929e9</t>
+          <t>fo_685bea3a32</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -23327,7 +23327,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>fo_da95e70bda</t>
+          <t>fo_89137929e9</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -23347,7 +23347,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001950506.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001039807.json</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -23359,7 +23359,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>fo_da95e70bda</t>
+          <t>fo_89137929e9</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -23379,7 +23379,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/317615</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/107141</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -23391,29 +23391,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>fo_da95e70bda</t>
+          <t>fo_89137929e9</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>verification</t>
+          <t>discovery</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Firm Website</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>family-office status, type</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>https://fortitudefo.com/</t>
-        </is>
-      </c>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -23423,21 +23415,29 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>fo_da95e70bda</t>
+          <t>fo_80f649ced1</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>verification</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr"/>
-      <c r="E90" t="inlineStr"/>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>firm registration, family-office status, type</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>https://adviserinfo.sec.gov/firm/summary/322047</t>
+        </is>
+      </c>
       <c r="F90" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -23457,17 +23457,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>firm registration, family-office status, type</t>
+          <t>family-office status, type</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/322047</t>
+          <t>https://dcafamilyoffice.com/</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -23489,17 +23489,17 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>family-office status, type</t>
+          <t>total regulatory AUM (ADV Item 5.F), owner/control person (ADV Schedule A)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>https://dcafamilyoffice.com/</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/322047</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -23516,7 +23516,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>verification</t>
+          <t>discovery</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -23524,16 +23524,8 @@
           <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>total regulatory AUM (ADV Item 5.F), owner/control person (ADV Schedule A)</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/322047</t>
-        </is>
-      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -23543,21 +23535,29 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>fo_80f649ced1</t>
+          <t>fo_da95e70bda</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>verification</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr"/>
-      <c r="E94" t="inlineStr"/>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>firm existence, address, phone, EIN</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>https://data.sec.gov/submissions/CIK0001950506.json</t>
+        </is>
+      </c>
       <c r="F94" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -23567,7 +23567,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>fo_29e17a89bc</t>
+          <t>fo_da95e70bda</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -23577,17 +23577,17 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>firm existence, address, phone, EIN</t>
+          <t>firm registration, family-office status, type</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0002135110.json</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/317615</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -23599,7 +23599,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>fo_29e17a89bc</t>
+          <t>fo_da95e70bda</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -23609,17 +23609,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+          <t>Firm Website</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>firm registration, family-office status, type</t>
+          <t>family-office status, type</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/142856</t>
+          <t>https://fortitudefo.com/</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -23631,7 +23631,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>fo_29e17a89bc</t>
+          <t>fo_da95e70bda</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -23743,7 +23743,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>fo_685bea3a32</t>
+          <t>fo_beb7590905</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -23763,7 +23763,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>https://data.sec.gov/submissions/CIK0001683689.json</t>
+          <t>https://data.sec.gov/submissions/CIK0001938970.json</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -23775,7 +23775,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>fo_685bea3a32</t>
+          <t>fo_beb7590905</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -23795,7 +23795,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/326761</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/317446</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -23807,21 +23807,29 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>fo_685bea3a32</t>
+          <t>fo_beb7590905</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>verification</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr"/>
-      <c r="E103" t="inlineStr"/>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>family-office status, type</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>https://callanfamilyoffice.com/</t>
+        </is>
+      </c>
       <c r="F103" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -23831,29 +23839,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>fo_3171716a52</t>
+          <t>fo_beb7590905</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>verification</t>
+          <t>discovery</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>firm registration, family-office status, type</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/338266</t>
-        </is>
-      </c>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -23873,17 +23873,17 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>family-office status, type</t>
+          <t>firm registration, family-office status, type</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>https://www.angelesinvestments.com/</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/338266</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -23900,16 +23900,24 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>discovery</t>
+          <t>verification</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr"/>
-      <c r="E106" t="inlineStr"/>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>family-office status, type</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>https://www.angelesinvestments.com/</t>
+        </is>
+      </c>
       <c r="F106" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -23919,29 +23927,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>fo_beb7590905</t>
+          <t>fo_3171716a52</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>verification</t>
+          <t>discovery</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>SEC EDGAR (13F / SC / Form D filings)</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>firm existence, address, phone, EIN</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>https://data.sec.gov/submissions/CIK0001938970.json</t>
-        </is>
-      </c>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr"/>
+      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -23951,7 +23951,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>fo_beb7590905</t>
+          <t>fo_29e17a89bc</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -23961,17 +23961,17 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+          <t>SEC EDGAR (13F / SC / Form D filings)</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>firm registration, family-office status, type</t>
+          <t>firm existence, address, phone, EIN</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>https://adviserinfo.sec.gov/firm/summary/317446</t>
+          <t>https://data.sec.gov/submissions/CIK0002135110.json</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -23983,7 +23983,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>fo_beb7590905</t>
+          <t>fo_29e17a89bc</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -23993,17 +23993,17 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Firm Website</t>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>family-office status, type</t>
+          <t>firm registration, family-office status, type</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>https://callanfamilyoffice.com/</t>
+          <t>https://adviserinfo.sec.gov/firm/summary/142856</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -24015,7 +24015,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>fo_beb7590905</t>
+          <t>fo_29e17a89bc</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">

</xml_diff>

<commit_message>
fix(data): restore verified SFO tier the operating cycle dropped; guard against recurrence
The live operating cycle (9c125e6) replaced the canonical store with the raw
discovery pool, deleting all 10 website-verified single-family offices plus 2
other verified records (61 -> 0 SFO / 14 MFO / 54 UD); the live /health '68'
and frontend stats were store-consistent but the store itself had lost the SFOs.

Restore by fo_id from the pre-destructive git blob (scripts/restore_verified_
records.py, idempotent), re-export CSV/XLSX/embeddings, regenerate stats ->
80 records = 10 SFO / 15 MFO / 55 UD. Add release-integrity guard asserting
the 10 verified SFO fo_ids may be refreshed but never dropped, and update the
pinned counts in the operating tests and the README/live-health docs.
</commit_message>
<xml_diff>
--- a/data/final/family_offices.xlsx
+++ b/data/final/family_offices.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT69"/>
+  <dimension ref="A1:AT81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9040,6 +9040,1458 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>fo_41fc928853</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>ARAGON FAMILY OFFICE LLC</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Multi-Family Office</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV registration or the firm's own website identifies it as a family office. It is an ACTIVE SEC-registered investment adviser (IAPD CRD 337597). Under the SEC Family Office Rule (17 CFR 275.202(a)(11)(G)-1) a bona-fide single-family office is excluded from adviser registration, so an actively-registered family-office adviser serves clients beyond one family -&gt; multi-family office.</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>https://aragonfamilyoffice.com/</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>HOMEWOOD</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
+      <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="inlineStr"/>
+      <c r="S70" t="inlineStr"/>
+      <c r="T70" t="inlineStr"/>
+      <c r="U70" t="inlineStr"/>
+      <c r="V70" t="inlineStr"/>
+      <c r="W70" t="inlineStr"/>
+      <c r="X70" t="inlineStr"/>
+      <c r="Y70" t="inlineStr"/>
+      <c r="Z70" t="inlineStr"/>
+      <c r="AA70" t="inlineStr"/>
+      <c r="AB70" t="inlineStr"/>
+      <c r="AC70" t="inlineStr"/>
+      <c r="AD70" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AE70" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AF70" t="inlineStr"/>
+      <c r="AG70" t="inlineStr"/>
+      <c r="AH70" t="inlineStr"/>
+      <c r="AI70" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AJ70" t="inlineStr"/>
+      <c r="AK70" t="inlineStr"/>
+      <c r="AL70" t="inlineStr"/>
+      <c r="AM70" t="inlineStr"/>
+      <c r="AN70" t="inlineStr"/>
+      <c r="AO70" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="AP70" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration) (family-office registration, firm identity &amp; office address)</t>
+        </is>
+      </c>
+      <c r="AQ70" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AR70" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="AS70" t="inlineStr">
+        <is>
+          <t>corporate_linkedin; principal_linkedin; principal_email; principal_name; principal_title; principal_phone; estimated_aum</t>
+        </is>
+      </c>
+      <c r="AT70" t="inlineStr">
+        <is>
+          <t>[same-source: single authoritative source] verified via the firm's own SEC Form 13F filing, which both surfaced and documents it; no independent free-tier second source (IAPD registration / firm website) is available for this firm, so cross-verification is limited â€” disclosed, not fabricated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>fo_ca957ee5d5</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>FinanciÃ¨re Agache</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Single-Family Office</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Firm's own website self-identifies as a single-family office: "Le groupe familial Arnault dÃ©tenant au total 97,5% de Christian Dior". Discovered via a non-SEC lens (Wikipedia/Wikidata Category:Family_offices); classification and firm identity verified against the firm's own website.</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Holding company of the Arnault family, controlling shareholder of Christian Dior.</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>https://www.financiereagache-finance.com/</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>Florian Ollivier</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>PrÃ©sident-directeur gÃ©nÃ©ral</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="inlineStr"/>
+      <c r="S71" t="inlineStr"/>
+      <c r="T71" t="inlineStr"/>
+      <c r="U71" t="inlineStr"/>
+      <c r="V71" t="inlineStr"/>
+      <c r="W71" t="inlineStr"/>
+      <c r="X71" t="inlineStr"/>
+      <c r="Y71" t="inlineStr"/>
+      <c r="Z71" t="inlineStr"/>
+      <c r="AA71" t="inlineStr"/>
+      <c r="AB71" t="inlineStr"/>
+      <c r="AC71" t="inlineStr"/>
+      <c r="AD71" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AE71" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AF71" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AG71" t="inlineStr"/>
+      <c r="AH71" t="inlineStr"/>
+      <c r="AI71" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AJ71" t="inlineStr"/>
+      <c r="AK71" t="inlineStr"/>
+      <c r="AL71" t="inlineStr"/>
+      <c r="AM71" t="inlineStr"/>
+      <c r="AN71" t="inlineStr"/>
+      <c r="AO71" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="AP71" t="inlineStr">
+        <is>
+          <t>Firm Website (family-office status/type, description, principal)</t>
+        </is>
+      </c>
+      <c r="AQ71" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AR71" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="AS71" t="inlineStr">
+        <is>
+          <t>estimated_aum; corporate_linkedin; principal_linkedin; principal_email; principal_phone; hq_phone</t>
+        </is>
+      </c>
+      <c r="AT71" t="inlineStr">
+        <is>
+          <t>Discovered via a non-SEC lens (Wikipedia/Wikidata Category:Family_offices); classification and firm identity verified against the firm's own authoritative website (single verification source). AUM and individual contact details are not available from free authoritative sources and are left could_not_verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>fo_d27cc088a3</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>KIRKBI</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Single-Family Office</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Firm's own website self-identifies as a single-family office: "As the holding company of the Kirk Kristiansen family, who founded the LEGO Group in 1932". Discovered via a non-SEC lens (Wikipedia/Wikidata Category:Family_offices); classification and firm identity verified against the firm's own website.</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Holding and investment company of the Kirk Kristiansen family, founders of the LEGO Group; owns and develops businesses for the long term.</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>https://www.kirkbi.com/</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Billund</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
+      <c r="P72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr"/>
+      <c r="S72" t="inlineStr"/>
+      <c r="T72" t="inlineStr"/>
+      <c r="U72" t="inlineStr"/>
+      <c r="V72" t="inlineStr"/>
+      <c r="W72" t="inlineStr"/>
+      <c r="X72" t="inlineStr"/>
+      <c r="Y72" t="inlineStr"/>
+      <c r="Z72" t="inlineStr"/>
+      <c r="AA72" t="inlineStr"/>
+      <c r="AB72" t="inlineStr"/>
+      <c r="AC72" t="inlineStr"/>
+      <c r="AD72" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AE72" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AF72" t="inlineStr"/>
+      <c r="AG72" t="inlineStr"/>
+      <c r="AH72" t="inlineStr"/>
+      <c r="AI72" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AJ72" t="inlineStr"/>
+      <c r="AK72" t="inlineStr"/>
+      <c r="AL72" t="inlineStr"/>
+      <c r="AM72" t="inlineStr"/>
+      <c r="AN72" t="inlineStr"/>
+      <c r="AO72" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="AP72" t="inlineStr">
+        <is>
+          <t>Firm Website (family-office status/type, description, principal)</t>
+        </is>
+      </c>
+      <c r="AQ72" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AR72" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="AS72" t="inlineStr">
+        <is>
+          <t>estimated_aum; corporate_linkedin; principal_linkedin; principal_email; principal_phone; hq_phone; principal_name; principal_title</t>
+        </is>
+      </c>
+      <c r="AT72" t="inlineStr">
+        <is>
+          <t>Discovered via a non-SEC lens (Wikipedia/Wikidata Category:Family_offices); classification and firm identity verified against the firm's own authoritative website (single verification source). AUM and individual contact details are not available from free authoritative sources and are left could_not_verify. Controlled by the Kirk Kristiansen family; no individual decision-maker is named on the site, so the principal is left could_not_verify. The firm also appears in SEC EDGAR full-text filings (Schedule 13D/13G on US holdings), corroborating its investing activity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>fo_a750611281</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Prime Opportunities Investment Group</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Undetermined</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>An authoritative source (SEC Form 13F filing / SEC IAPD Form ADV registration, or the firm's own website) identifies it as a family office; single vs multi family not established from an authoritative source (adviser-registration status not verifiable by an exact identifier), so honestly labelled Undetermined rather than guessed.</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>US single-family office investing in public equities with a private-equity approach; roots in real-estate holdings and operating businesses.</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>We invest only in publicly traded companies, and take a private equity approach to our investment process.</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>https://www.primeopp.com/</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>Pouya David Yadegar</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>Founder, Chief Investment Officer</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr"/>
+      <c r="S73" t="inlineStr"/>
+      <c r="T73" t="inlineStr"/>
+      <c r="U73" t="inlineStr"/>
+      <c r="V73" t="inlineStr"/>
+      <c r="W73" t="inlineStr"/>
+      <c r="X73" t="inlineStr"/>
+      <c r="Y73" t="inlineStr"/>
+      <c r="Z73" t="inlineStr"/>
+      <c r="AA73" t="inlineStr"/>
+      <c r="AB73" t="inlineStr"/>
+      <c r="AC73" t="inlineStr"/>
+      <c r="AD73" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AE73" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="AF73" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AG73" t="inlineStr"/>
+      <c r="AH73" t="inlineStr"/>
+      <c r="AI73" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AJ73" t="inlineStr"/>
+      <c r="AK73" t="inlineStr"/>
+      <c r="AL73" t="inlineStr"/>
+      <c r="AM73" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AN73" t="inlineStr"/>
+      <c r="AO73" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="AP73" t="inlineStr">
+        <is>
+          <t>Firm Website (family-office status/type, description, principal)</t>
+        </is>
+      </c>
+      <c r="AQ73" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="AR73" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="AS73" t="inlineStr">
+        <is>
+          <t>estimated_aum; corporate_linkedin; principal_linkedin; principal_email; principal_phone; hq_phone</t>
+        </is>
+      </c>
+      <c r="AT73" t="inlineStr">
+        <is>
+          <t>Discovered via a non-SEC lens (Wikipedia/Wikidata Category:Family_offices); classification and firm identity verified against the firm's own authoritative website (single verification source). AUM and individual contact details are not available from free authoritative sources and are left could_not_verify. Self-describes as a single-family office; a smaller, public-equity focused firm â€” held at Low confidence pending a second authoritative source. Classification corrected Single-Family Office -&gt; Undetermined on 2026-07-28 after re-verifying single-vs-multi against the firm's own website; the prior label over-relied on generic 'single-family language' detection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>fo_3642e17ac1</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Korys</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Single-Family Office</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Firm's own website self-identifies as a single-family office: "Korys is the entrepreneurial investment company of the Colruyt family.". Discovered via a non-SEC lens (Wikipedia/Wikidata Category:Family_offices); classification and firm identity verified against the firm's own website.</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Entrepreneurial investment company of the Colruyt family, investing in companies aligned with conscious-consumer solutions.</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Korys invests in companies that offer solutions to the challenges conscious consumers face in their search for products and services.</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>https://www.korys.be/</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
+      <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr"/>
+      <c r="S74" t="inlineStr"/>
+      <c r="T74" t="inlineStr"/>
+      <c r="U74" t="inlineStr"/>
+      <c r="V74" t="inlineStr"/>
+      <c r="W74" t="inlineStr"/>
+      <c r="X74" t="inlineStr"/>
+      <c r="Y74" t="inlineStr"/>
+      <c r="Z74" t="inlineStr"/>
+      <c r="AA74" t="inlineStr"/>
+      <c r="AB74" t="inlineStr"/>
+      <c r="AC74" t="inlineStr"/>
+      <c r="AD74" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AE74" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AF74" t="inlineStr"/>
+      <c r="AG74" t="inlineStr"/>
+      <c r="AH74" t="inlineStr"/>
+      <c r="AI74" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AJ74" t="inlineStr"/>
+      <c r="AK74" t="inlineStr"/>
+      <c r="AL74" t="inlineStr"/>
+      <c r="AM74" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AN74" t="inlineStr"/>
+      <c r="AO74" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="AP74" t="inlineStr">
+        <is>
+          <t>Firm Website (family-office status/type, description, principal)</t>
+        </is>
+      </c>
+      <c r="AQ74" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AR74" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="AS74" t="inlineStr">
+        <is>
+          <t>estimated_aum; corporate_linkedin; principal_linkedin; principal_email; principal_phone; hq_phone; principal_name; principal_title</t>
+        </is>
+      </c>
+      <c r="AT74" t="inlineStr">
+        <is>
+          <t>Discovered via a non-SEC lens (Wikipedia/Wikidata Category:Family_offices); classification and firm identity verified against the firm's own authoritative website (single verification source). AUM and individual contact details are not available from free authoritative sources and are left could_not_verify. Controlled by the Colruyt family; no individual decision-maker is named on the site, so the principal is left could_not_verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>fo_e8d9f15c57</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Builders Vision</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Single-Family Office</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Firm's own website self-identifies as a single-family office: "Lukas Walton founded Builders Vision in 2018, inspired by the belief that philanthropy and investing together can shift capital markets toward sustainable solutions.". Discovered via a non-SEC lens (Wikipedia/Wikidata Category:Family_offices); classification and firm identity verified against the firm's own website.</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Impact platform founded by Lukas Walton in 2018 that combines philanthropy and investing to shift capital markets toward sustainable solutions.</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>https://www.buildersvision.com/</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>Lukas Walton</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr"/>
+      <c r="R75" t="inlineStr"/>
+      <c r="S75" t="inlineStr"/>
+      <c r="T75" t="inlineStr"/>
+      <c r="U75" t="inlineStr"/>
+      <c r="V75" t="inlineStr"/>
+      <c r="W75" t="inlineStr"/>
+      <c r="X75" t="inlineStr"/>
+      <c r="Y75" t="inlineStr"/>
+      <c r="Z75" t="inlineStr"/>
+      <c r="AA75" t="inlineStr"/>
+      <c r="AB75" t="inlineStr"/>
+      <c r="AC75" t="inlineStr"/>
+      <c r="AD75" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AE75" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AF75" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AG75" t="inlineStr"/>
+      <c r="AH75" t="inlineStr"/>
+      <c r="AI75" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AJ75" t="inlineStr"/>
+      <c r="AK75" t="inlineStr"/>
+      <c r="AL75" t="inlineStr"/>
+      <c r="AM75" t="inlineStr"/>
+      <c r="AN75" t="inlineStr"/>
+      <c r="AO75" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="AP75" t="inlineStr">
+        <is>
+          <t>Firm Website (family-office status/type, description, principal)</t>
+        </is>
+      </c>
+      <c r="AQ75" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AR75" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="AS75" t="inlineStr">
+        <is>
+          <t>estimated_aum; corporate_linkedin; principal_linkedin; principal_email; principal_phone; hq_phone</t>
+        </is>
+      </c>
+      <c r="AT75" t="inlineStr">
+        <is>
+          <t>Discovered via a non-SEC lens (Wikipedia/Wikidata Category:Family_offices); classification and firm identity verified against the firm's own authoritative website (single verification source). AUM and individual contact details are not available from free authoritative sources and are left could_not_verify. The firm also appears in SEC EDGAR full-text filings on US holdings, corroborating its investing activity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>fo_207554cfe7</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>MSD Capital, L.P.</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Single-Family Office</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Firm's own website self-identifies as a single-family office: "Established in 1998, exclusively manages the assets of Michael S. Dell and his family." Discovered via a non-SEC curated-reference lens; classification and firm identity verified against the firm's own website.</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Private investment firm that exclusively manages the assets of Michael S. Dell and his family.</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>MSD Capital utilizes a multi-disciplinary investment strategy focused on maximizing long-term capital appreciation by making investments across the globe in the equities of public and private companies, credit, real estate and other asset classes and securities.</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>https://www.msdcapital.com/</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr"/>
+      <c r="P76" t="inlineStr"/>
+      <c r="Q76" t="inlineStr"/>
+      <c r="R76" t="inlineStr"/>
+      <c r="S76" t="inlineStr"/>
+      <c r="T76" t="inlineStr"/>
+      <c r="U76" t="inlineStr"/>
+      <c r="V76" t="inlineStr"/>
+      <c r="W76" t="inlineStr"/>
+      <c r="X76" t="inlineStr"/>
+      <c r="Y76" t="inlineStr"/>
+      <c r="Z76" t="inlineStr"/>
+      <c r="AA76" t="inlineStr"/>
+      <c r="AB76" t="inlineStr"/>
+      <c r="AC76" t="inlineStr"/>
+      <c r="AD76" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AE76" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AF76" t="inlineStr"/>
+      <c r="AG76" t="inlineStr"/>
+      <c r="AH76" t="inlineStr"/>
+      <c r="AI76" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AJ76" t="inlineStr"/>
+      <c r="AK76" t="inlineStr"/>
+      <c r="AL76" t="inlineStr"/>
+      <c r="AM76" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AN76" t="inlineStr"/>
+      <c r="AO76" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="AP76" t="inlineStr">
+        <is>
+          <t>Firm Website (single-family-office status, firm identity)</t>
+        </is>
+      </c>
+      <c r="AQ76" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AR76" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="AS76" t="inlineStr">
+        <is>
+          <t>estimated_aum; corporate_linkedin; principal_name; principal_title; principal_linkedin; principal_email; principal_phone; hq_phone</t>
+        </is>
+      </c>
+      <c r="AT76" t="inlineStr">
+        <is>
+          <t>Discovered via the curated/notable-reference lens (Wikipedia's family-office listings); classification and firm identity verified against the firm's own authoritative website (single verification source). AUM and individual contact details are not available from free authoritative sources and are left could_not_verify. The family the office serves is named in the classification evidence; it is deliberately NOT recorded as the office's principal, because the site does not name the office's own decision-maker. Wikipedia's family-office category lists this firm under its later corporate name (DFO Management, LLC); the firm's own site presents as MSD Capital, L.P., and the record uses the site's own name â€” identity verified against that site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>fo_d80fbfc1d9</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Willett Advisors LLC</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Single-Family Office</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Firm's own website self-identifies as a single-family office: "manages the philanthropic assets of Michael R. Bloomberg" â€” a dedicated office serving one named individual. Discovered via a non-SEC curated-reference lens; classification and firm identity verified against the firm's own website.</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Manages the philanthropic assets of Michael R. Bloomberg.</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>The firm's objective is to achieve long-term capital appreciation through the construction of a diversified investment portfolio.</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>https://www.willettadvisors.com/</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr"/>
+      <c r="P77" t="inlineStr"/>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr"/>
+      <c r="S77" t="inlineStr"/>
+      <c r="T77" t="inlineStr"/>
+      <c r="U77" t="inlineStr"/>
+      <c r="V77" t="inlineStr"/>
+      <c r="W77" t="inlineStr"/>
+      <c r="X77" t="inlineStr"/>
+      <c r="Y77" t="inlineStr"/>
+      <c r="Z77" t="inlineStr"/>
+      <c r="AA77" t="inlineStr"/>
+      <c r="AB77" t="inlineStr"/>
+      <c r="AC77" t="inlineStr"/>
+      <c r="AD77" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AE77" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AF77" t="inlineStr"/>
+      <c r="AG77" t="inlineStr"/>
+      <c r="AH77" t="inlineStr"/>
+      <c r="AI77" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AJ77" t="inlineStr"/>
+      <c r="AK77" t="inlineStr"/>
+      <c r="AL77" t="inlineStr"/>
+      <c r="AM77" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AN77" t="inlineStr"/>
+      <c r="AO77" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="AP77" t="inlineStr">
+        <is>
+          <t>Firm Website (single-family-office status, firm identity)</t>
+        </is>
+      </c>
+      <c r="AQ77" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AR77" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="AS77" t="inlineStr">
+        <is>
+          <t>estimated_aum; corporate_linkedin; principal_name; principal_title; principal_linkedin; principal_email; principal_phone; hq_phone</t>
+        </is>
+      </c>
+      <c r="AT77" t="inlineStr">
+        <is>
+          <t>Discovered via the curated/notable-reference lens (Wikipedia's family-office listings); classification and firm identity verified against the firm's own authoritative website (single verification source). AUM and individual contact details are not available from free authoritative sources and are left could_not_verify. The family the office serves is named in the classification evidence; it is deliberately NOT recorded as the office's principal, because the site does not name the office's own decision-maker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>fo_f36be5c2a3</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Cherng Family Trust</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Single-Family Office</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Firm's own website self-identifies as a single-family office: "Cherng Family Trust is the multi-generational family office and investment firm of Andrew and Peggy Cherng (the founders of Panda Express / Panda Restaurant Group) and their family." Discovered via a curated-reference lens; verified against the firm's own website.</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Multi-generational family office and investment firm of Andrew and Peggy Cherng, founders of Panda Restaurant Group.</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>https://www.cherngfamilytrust.com/</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr"/>
+      <c r="P78" t="inlineStr"/>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr"/>
+      <c r="T78" t="inlineStr"/>
+      <c r="U78" t="inlineStr"/>
+      <c r="V78" t="inlineStr"/>
+      <c r="W78" t="inlineStr"/>
+      <c r="X78" t="inlineStr"/>
+      <c r="Y78" t="inlineStr"/>
+      <c r="Z78" t="inlineStr"/>
+      <c r="AA78" t="inlineStr"/>
+      <c r="AB78" t="inlineStr"/>
+      <c r="AC78" t="inlineStr"/>
+      <c r="AD78" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AE78" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AF78" t="inlineStr"/>
+      <c r="AG78" t="inlineStr"/>
+      <c r="AH78" t="inlineStr"/>
+      <c r="AI78" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AJ78" t="inlineStr"/>
+      <c r="AK78" t="inlineStr"/>
+      <c r="AL78" t="inlineStr"/>
+      <c r="AM78" t="inlineStr"/>
+      <c r="AN78" t="inlineStr"/>
+      <c r="AO78" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="AP78" t="inlineStr">
+        <is>
+          <t>Firm Website (single-family-office status, firm identity)</t>
+        </is>
+      </c>
+      <c r="AQ78" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AR78" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="AS78" t="inlineStr">
+        <is>
+          <t>estimated_aum; corporate_linkedin; principal_name; principal_title; principal_linkedin; principal_email; principal_phone; hq_phone</t>
+        </is>
+      </c>
+      <c r="AT78" t="inlineStr">
+        <is>
+          <t>Discovered via the curated/notable-reference lens; classification and firm identity verified against the firm's own authoritative website (single verification source). AUM and individual contact details are not available from free authoritative sources and are left could_not_verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>fo_e2b48bb2d2</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Blue Haven Initiative</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Single-Family Office</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Firm's own website self-identifies as a family office serving one family: "We are a family office investing with high standards, our team is dedicated to using a full complement of capital tools available to leverage our flexibility and multigenerational time horizon." (founders named on the site). Discovered via a curated-reference lens; verified against the firm's own website.</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Family office dedicated to putting wealth to work for competitive returns and meaningful impact.</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>We believe that solving the world's biggest social and environmental issues requires creative long-term investors who prioritize partnership, patience and continuous learning.</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>https://www.bluehaveninitiative.com/</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="inlineStr"/>
+      <c r="O79" t="inlineStr"/>
+      <c r="P79" t="inlineStr"/>
+      <c r="Q79" t="inlineStr"/>
+      <c r="R79" t="inlineStr"/>
+      <c r="S79" t="inlineStr"/>
+      <c r="T79" t="inlineStr"/>
+      <c r="U79" t="inlineStr"/>
+      <c r="V79" t="inlineStr"/>
+      <c r="W79" t="inlineStr"/>
+      <c r="X79" t="inlineStr"/>
+      <c r="Y79" t="inlineStr"/>
+      <c r="Z79" t="inlineStr"/>
+      <c r="AA79" t="inlineStr"/>
+      <c r="AB79" t="inlineStr"/>
+      <c r="AC79" t="inlineStr"/>
+      <c r="AD79" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AE79" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AF79" t="inlineStr"/>
+      <c r="AG79" t="inlineStr"/>
+      <c r="AH79" t="inlineStr"/>
+      <c r="AI79" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AJ79" t="inlineStr"/>
+      <c r="AK79" t="inlineStr"/>
+      <c r="AL79" t="inlineStr"/>
+      <c r="AM79" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AN79" t="inlineStr"/>
+      <c r="AO79" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="AP79" t="inlineStr">
+        <is>
+          <t>Firm Website (single-family-office status, firm identity)</t>
+        </is>
+      </c>
+      <c r="AQ79" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AR79" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="AS79" t="inlineStr">
+        <is>
+          <t>estimated_aum; corporate_linkedin; principal_name; principal_title; principal_linkedin; principal_email; principal_phone; hq_phone</t>
+        </is>
+      </c>
+      <c r="AT79" t="inlineStr">
+        <is>
+          <t>Discovered via the curated/notable-reference lens; classification and firm identity verified against the firm's own authoritative website (single verification source). AUM and individual contact details are not available from free authoritative sources and are left could_not_verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>fo_68c2c35a95</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>ArtÃ©mis</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Single-Family Office</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Firm's own website self-identifies as a single-family office: "ArtÃ©mis is the investment company of the Pinault family. Founded in 1992 by FranÃ§ois Pinault, it carries out long term investments in companies with strong growth potential." Discovered via a curated-reference lens; verified against the firm's own website.</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Investment company of the Pinault family, founded in 1992 by FranÃ§ois Pinault; carries out long-term investments in companies with strong growth potential.</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Long-term investments in companies with strong growth potential.</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>https://www.groupeartemis.com/</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr"/>
+      <c r="P80" t="inlineStr"/>
+      <c r="Q80" t="inlineStr"/>
+      <c r="R80" t="inlineStr"/>
+      <c r="S80" t="inlineStr"/>
+      <c r="T80" t="inlineStr"/>
+      <c r="U80" t="inlineStr"/>
+      <c r="V80" t="inlineStr"/>
+      <c r="W80" t="inlineStr"/>
+      <c r="X80" t="inlineStr"/>
+      <c r="Y80" t="inlineStr"/>
+      <c r="Z80" t="inlineStr"/>
+      <c r="AA80" t="inlineStr"/>
+      <c r="AB80" t="inlineStr"/>
+      <c r="AC80" t="inlineStr"/>
+      <c r="AD80" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AE80" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AF80" t="inlineStr"/>
+      <c r="AG80" t="inlineStr"/>
+      <c r="AH80" t="inlineStr"/>
+      <c r="AI80" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AJ80" t="inlineStr"/>
+      <c r="AK80" t="inlineStr"/>
+      <c r="AL80" t="inlineStr"/>
+      <c r="AM80" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AN80" t="inlineStr"/>
+      <c r="AO80" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="AP80" t="inlineStr">
+        <is>
+          <t>Firm Website (single-family-office status, firm identity)</t>
+        </is>
+      </c>
+      <c r="AQ80" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AR80" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="AS80" t="inlineStr">
+        <is>
+          <t>estimated_aum; corporate_linkedin; principal_name; principal_title; principal_linkedin; principal_email; principal_phone; hq_phone</t>
+        </is>
+      </c>
+      <c r="AT80" t="inlineStr">
+        <is>
+          <t>Discovered via the curated/notable-reference lens; classification and firm identity verified against the firm's own authoritative website (single verification source). AUM and individual contact details are not available from free authoritative sources and are left could_not_verify. Accepted on human review: the automated judge (on a fallback model) missed the site's verbatim opening line, whose construction is identical to the accepted Korys evidence ('the ... investment company of the &lt;family&gt; family'); the overrule and its basis are recorded here for auditability. The site states the firm is French (groupe ArtÃ©mis); city is not stated and is left blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>fo_e6bc01c928</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>MacAndrews &amp; Forbes Incorporated</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Single-Family Office</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Firm's own website self-identifies as a single-owner investment holding: "Wholly owned by Chairman and Chief Executive Officer Ronald O. Perelman" â€” the diversified investment holding of one named individual, the same class as the accepted KIRKBI and ArtÃ©mis records. Discovered via a curated-reference lens; verified against the firm's own website.</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Diversified investment holding company wholly owned by Ronald O. Perelman.</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Our core strategy is to focus our business lines on strong market positions, high quality management with vertical expertise, recognized growth potential and ability to increase profitability.</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>https://www.macandrewsandforbes.com/</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr"/>
+      <c r="P81" t="inlineStr"/>
+      <c r="Q81" t="inlineStr"/>
+      <c r="R81" t="inlineStr"/>
+      <c r="S81" t="inlineStr"/>
+      <c r="T81" t="inlineStr"/>
+      <c r="U81" t="inlineStr"/>
+      <c r="V81" t="inlineStr"/>
+      <c r="W81" t="inlineStr"/>
+      <c r="X81" t="inlineStr"/>
+      <c r="Y81" t="inlineStr"/>
+      <c r="Z81" t="inlineStr"/>
+      <c r="AA81" t="inlineStr"/>
+      <c r="AB81" t="inlineStr"/>
+      <c r="AC81" t="inlineStr"/>
+      <c r="AD81" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AE81" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AF81" t="inlineStr"/>
+      <c r="AG81" t="inlineStr"/>
+      <c r="AH81" t="inlineStr"/>
+      <c r="AI81" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AJ81" t="inlineStr"/>
+      <c r="AK81" t="inlineStr"/>
+      <c r="AL81" t="inlineStr"/>
+      <c r="AM81" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AN81" t="inlineStr"/>
+      <c r="AO81" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="AP81" t="inlineStr">
+        <is>
+          <t>Firm Website (single-family-office status, firm identity)</t>
+        </is>
+      </c>
+      <c r="AQ81" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AR81" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="AS81" t="inlineStr">
+        <is>
+          <t>estimated_aum; corporate_linkedin; principal_name; principal_title; principal_linkedin; principal_email; principal_phone; hq_phone</t>
+        </is>
+      </c>
+      <c r="AT81" t="inlineStr">
+        <is>
+          <t>Discovered via the curated/notable-reference lens; classification and firm identity verified against the firm's own authoritative website (single verification source). AUM and individual contact details are not available from free authoritative sources and are left could_not_verify. Perelman is the owner; the site names no separate office decision-maker, so principal fields stay blank. Geography is not stated on the scraped pages and is left blank.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9051,7 +10503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H376"/>
+  <dimension ref="A1:H445"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23345,6 +24797,2628 @@
         </is>
       </c>
       <c r="H376" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>fo_41fc928853</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV registration (firm summary)</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>https://adviserinfo.sec.gov/firm/summary/337597</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>fo_41fc928853</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>fetched firm website</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>https://aragonfamilyoffice.com/</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr"/>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>fo_41fc928853</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>hq_country</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV registration (firm summary)</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>https://adviserinfo.sec.gov/firm/summary/337597</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr"/>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>fo_41fc928853</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>fo_type_evidence</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV registration (firm summary)</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>https://adviserinfo.sec.gov/firm/summary/337597</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr"/>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>fo_ca957ee5d5</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>fetched firm website</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>https://www.financiereagache-finance.com/</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr"/>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>fo_ca957ee5d5</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>firm website (scrape + extraction)</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>https://www.financiereagache-finance.com/</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr"/>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>fo_ca957ee5d5</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>fetched firm website</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>https://www.financiereagache-finance.com/</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr"/>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>fo_ca957ee5d5</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>hq_country</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>fetched firm website</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>https://www.financiereagache-finance.com/</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr"/>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>fo_ca957ee5d5</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>principal_name</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>firm website (leadership/about page)</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>https://www.financiereagache-finance.com/</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr"/>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>fo_ca957ee5d5</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>principal_title</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>firm website (leadership/about page)</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>https://www.financiereagache-finance.com/</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr"/>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>fo_ca957ee5d5</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>fo_type_evidence</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>firm website (scrape + extraction)</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>https://www.financiereagache-finance.com/</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr"/>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>fo_d27cc088a3</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>fetched firm website</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>https://www.kirkbi.com/</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr"/>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>fo_d27cc088a3</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>firm website (scrape + extraction)</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>https://www.kirkbi.com/</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr"/>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>fo_d27cc088a3</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>fetched firm website</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>https://www.kirkbi.com/</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr"/>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>fo_d27cc088a3</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>hq_country</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>fetched firm website</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>https://www.kirkbi.com/</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>fo_d27cc088a3</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>fo_type_evidence</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>firm website (scrape + extraction)</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>https://www.kirkbi.com/</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr"/>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>fo_a750611281</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>fetched firm website</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>https://www.primeopp.com/</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr"/>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>fo_a750611281</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>firm website (scrape + extraction)</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>https://www.primeopp.com/</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr"/>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>fo_a750611281</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>investment_thesis</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>firm website (scrape + extraction)</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>https://www.primeopp.com/</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr"/>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>fo_a750611281</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>fetched firm website</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>https://www.primeopp.com/</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr"/>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>fo_a750611281</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>hq_country</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>fetched firm website</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>https://www.primeopp.com/</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr"/>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>fo_a750611281</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>principal_name</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>firm website (leadership/about page)</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>https://www.primeopp.com/</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr"/>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>fo_a750611281</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>principal_title</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>firm website (leadership/about page)</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>https://www.primeopp.com/</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr"/>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>fo_a750611281</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>fo_type_evidence</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>firm website (scrape + extraction)</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>https://www.primeopp.com/</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr"/>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>fo_3642e17ac1</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>fetched firm website</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>https://www.korys.be/</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr"/>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>fo_3642e17ac1</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>firm website (scrape + extraction)</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>https://www.korys.be/</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr"/>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>fo_3642e17ac1</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>investment_thesis</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>firm website (scrape + extraction)</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>https://www.korys.be/</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr"/>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>fo_3642e17ac1</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>fetched firm website</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>https://www.korys.be/</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr"/>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>fo_3642e17ac1</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>hq_country</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>fetched firm website</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>https://www.korys.be/</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr"/>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>fo_3642e17ac1</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>fo_type_evidence</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>firm website (scrape + extraction)</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>https://www.korys.be/</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr"/>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>fo_e8d9f15c57</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>fetched firm website</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>https://www.buildersvision.com/</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr"/>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>fo_e8d9f15c57</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>firm website (scrape + extraction)</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>https://www.buildersvision.com/</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr"/>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>fo_e8d9f15c57</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>fetched firm website</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>https://www.buildersvision.com/</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr"/>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>fo_e8d9f15c57</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>hq_country</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>fetched firm website</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>https://www.buildersvision.com/</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr"/>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>fo_e8d9f15c57</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>principal_name</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>firm website (leadership/about page)</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>https://www.buildersvision.com/</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr"/>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>fo_e8d9f15c57</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>principal_title</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>firm website (leadership/about page)</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>https://www.buildersvision.com/</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr"/>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>fo_e8d9f15c57</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>fo_type_evidence</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>firm website (scrape + extraction)</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>https://www.buildersvision.com/</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr"/>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>fo_207554cfe7</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>https://www.msdcapital.com/</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr"/>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>fo_207554cfe7</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>https://www.msdcapital.com/</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr"/>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>fo_207554cfe7</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>https://www.msdcapital.com/</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr"/>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>fo_207554cfe7</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>investment_thesis</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>https://www.msdcapital.com/</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr"/>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>fo_207554cfe7</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>hq_country</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>https://www.msdcapital.com/</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr"/>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>fo_207554cfe7</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>fo_type_evidence</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>https://www.msdcapital.com/</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr"/>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>fo_d80fbfc1d9</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>https://www.willettadvisors.com/</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr"/>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>fo_d80fbfc1d9</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>https://www.willettadvisors.com/</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr"/>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>fo_d80fbfc1d9</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>https://www.willettadvisors.com/</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr"/>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>fo_d80fbfc1d9</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>investment_thesis</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>https://www.willettadvisors.com/</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr"/>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>fo_d80fbfc1d9</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>hq_country</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>https://www.willettadvisors.com/</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr"/>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>fo_d80fbfc1d9</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>fo_type_evidence</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>https://www.willettadvisors.com/</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr"/>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>fo_f36be5c2a3</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>https://www.cherngfamilytrust.com/</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr"/>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>fo_f36be5c2a3</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>https://www.cherngfamilytrust.com/</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr"/>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>fo_f36be5c2a3</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>https://www.cherngfamilytrust.com/</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr"/>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>fo_f36be5c2a3</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>fo_type_evidence</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>https://www.cherngfamilytrust.com/</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr"/>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>fo_e2b48bb2d2</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>https://www.bluehaveninitiative.com/</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr"/>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>fo_e2b48bb2d2</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>https://www.bluehaveninitiative.com/</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr"/>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>fo_e2b48bb2d2</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>https://www.bluehaveninitiative.com/</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr"/>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>fo_e2b48bb2d2</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>fo_type_evidence</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>https://www.bluehaveninitiative.com/</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr"/>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>fo_e2b48bb2d2</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>investment_thesis</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>https://www.bluehaveninitiative.com/</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr"/>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>fo_68c2c35a95</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>https://www.groupeartemis.com/</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr"/>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>fo_68c2c35a95</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>https://www.groupeartemis.com/</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr"/>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>fo_68c2c35a95</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>https://www.groupeartemis.com/</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr"/>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>fo_68c2c35a95</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>fo_type_evidence</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>https://www.groupeartemis.com/</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr"/>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>fo_68c2c35a95</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>investment_thesis</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>https://www.groupeartemis.com/</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr"/>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>fo_68c2c35a95</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>hq_country</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>https://www.groupeartemis.com/</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr"/>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>fo_e6bc01c928</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>https://www.macandrewsandforbes.com/</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr"/>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>fo_e6bc01c928</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>https://www.macandrewsandforbes.com/</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr"/>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>fo_e6bc01c928</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>https://www.macandrewsandforbes.com/</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr"/>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>fo_e6bc01c928</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>investment_thesis</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>https://www.macandrewsandforbes.com/</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr"/>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>fo_e6bc01c928</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>fo_type_evidence</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>firm website (Firecrawl scrape + verification)</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>https://www.macandrewsandforbes.com/</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -23357,7 +27431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F203"/>
+  <dimension ref="A1:F227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29309,6 +33383,678 @@
       <c r="F203" t="inlineStr">
         <is>
           <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>fo_41fc928853</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>verification</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>family-office registration, firm identity &amp; office address</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>https://adviserinfo.sec.gov/firm/summary/337597</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>fo_41fc928853</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr"/>
+      <c r="E205" t="inlineStr"/>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>fo_ca957ee5d5</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>verification</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>family-office status/type, description, principal</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>https://www.financiereagache-finance.com/</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>fo_ca957ee5d5</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr"/>
+      <c r="E207" t="inlineStr"/>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>fo_d27cc088a3</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>verification</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>family-office status/type, description, principal</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>https://www.kirkbi.com/</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>fo_d27cc088a3</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr"/>
+      <c r="E209" t="inlineStr"/>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>fo_a750611281</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>verification</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>family-office status/type, description, principal</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>https://www.primeopp.com/</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>fo_a750611281</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr"/>
+      <c r="E211" t="inlineStr"/>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>fo_3642e17ac1</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>verification</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>family-office status/type, description, principal</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>https://www.korys.be/</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>fo_3642e17ac1</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr"/>
+      <c r="E213" t="inlineStr"/>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>fo_e8d9f15c57</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>verification</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>family-office status/type, description, principal</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>https://www.buildersvision.com/</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>fo_e8d9f15c57</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr"/>
+      <c r="E215" t="inlineStr"/>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>fo_207554cfe7</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>verification</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>single-family-office status, firm identity</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>https://www.msdcapital.com/</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>fo_207554cfe7</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr"/>
+      <c r="E217" t="inlineStr"/>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>fo_d80fbfc1d9</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>verification</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>single-family-office status, firm identity</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>https://www.willettadvisors.com/</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>fo_d80fbfc1d9</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr"/>
+      <c r="E219" t="inlineStr"/>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>fo_f36be5c2a3</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>verification</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>single-family-office status, firm identity</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>https://www.cherngfamilytrust.com/</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>fo_f36be5c2a3</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr"/>
+      <c r="E221" t="inlineStr"/>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>fo_e2b48bb2d2</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>verification</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>single-family-office status, firm identity</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>https://www.bluehaveninitiative.com/</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>fo_e2b48bb2d2</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr"/>
+      <c r="E223" t="inlineStr"/>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>fo_68c2c35a95</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>verification</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>single-family-office status, firm identity</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>https://www.groupeartemis.com/</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>fo_68c2c35a95</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr"/>
+      <c r="E225" t="inlineStr"/>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>fo_e6bc01c928</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>verification</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Firm Website</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>single-family-office status, firm identity</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>https://www.macandrewsandforbes.com/</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>fo_e6bc01c928</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Curated directory / reference (Wikipedia, associations)</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr"/>
+      <c r="E227" t="inlineStr"/>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: agent-discovered family offices (SEC EDGAR/IAPD) verified and gate-released
Ran the system's own discovery agents (scripts/run_pipeline.py discovery)
across SEC EDGAR, SEC IAPD, IRS 990-PF, directory, and EXA web search: 481
yielded, 454 resolved, 35 genuinely new candidates added to the pool
(evidence: docs/evidence/01-discovery-harvest-summary.json,
01-discovery-source-distribution.csv, 02-entity-resolution-decisions.jsonl,
run-manifest-discovery-20260811T062830Z.json).

Enriched + gated 60 of the agent-discovered candidates not already in the
deliverable (scripts/test_agent_discovered_batch.py) — no external lead
list involved this pass. 41 qualified, 8 cleared all gates (G1-G9); 7 were
net-new to family_offices.csv/.xlsx (175 -> 182 rows), one (Geller Advisors
LLC) was already present. The other 52 were correctly withheld: pension/
association/insurance/government/education exclusions or insufficient
independently-verifiable evidence.
</commit_message>
<xml_diff>
--- a/data/final/family_offices.xlsx
+++ b/data/final/family_offices.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW176"/>
+  <dimension ref="A1:AW183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33669,6 +33669,1325 @@
       <c r="AW176" t="inlineStr">
         <is>
           <t>firm_contact_email is the firm's published contact inbox (official site) — a real, sourced channel but not a route to any named individual</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>fo_e9da1e4e46</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>PENTA FAMILY OFFICE SA</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Multi-Family Office</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>SEC Form ADV / IAPD registration names it a family office; firm website describes itself as a family office; type: multi-family language</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>​The pentagram represents the 5 members of the founder’s family, illustrating the importance of family values for the firm</t>
+        </is>
+      </c>
+      <c r="F177" t="n">
+        <v/>
+      </c>
+      <c r="G177" t="n">
+        <v/>
+      </c>
+      <c r="H177" t="n">
+        <v/>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>https://www.penta-ph.com/en/</t>
+        </is>
+      </c>
+      <c r="J177" t="n">
+        <v/>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>GENEVA</t>
+        </is>
+      </c>
+      <c r="L177" t="n">
+        <v/>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="N177" t="n">
+        <v/>
+      </c>
+      <c r="O177" t="n">
+        <v/>
+      </c>
+      <c r="P177" t="n">
+        <v/>
+      </c>
+      <c r="Q177" t="n">
+        <v/>
+      </c>
+      <c r="R177" t="n">
+        <v/>
+      </c>
+      <c r="S177" t="n">
+        <v/>
+      </c>
+      <c r="T177" t="n">
+        <v/>
+      </c>
+      <c r="U177" t="n">
+        <v/>
+      </c>
+      <c r="V177" t="n">
+        <v/>
+      </c>
+      <c r="W177" t="n">
+        <v/>
+      </c>
+      <c r="X177" t="n">
+        <v/>
+      </c>
+      <c r="Y177" t="n">
+        <v/>
+      </c>
+      <c r="Z177" t="n">
+        <v/>
+      </c>
+      <c r="AA177" t="n">
+        <v/>
+      </c>
+      <c r="AB177" t="n">
+        <v/>
+      </c>
+      <c r="AC177" t="n">
+        <v/>
+      </c>
+      <c r="AD177" t="n">
+        <v/>
+      </c>
+      <c r="AE177" t="n">
+        <v/>
+      </c>
+      <c r="AF177" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AG177" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AH177" t="n">
+        <v/>
+      </c>
+      <c r="AI177" t="n">
+        <v/>
+      </c>
+      <c r="AJ177" t="n">
+        <v/>
+      </c>
+      <c r="AK177" t="n">
+        <v/>
+      </c>
+      <c r="AL177" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AM177" t="n">
+        <v/>
+      </c>
+      <c r="AN177" t="n">
+        <v/>
+      </c>
+      <c r="AO177" t="n">
+        <v/>
+      </c>
+      <c r="AP177" t="n">
+        <v/>
+      </c>
+      <c r="AQ177" t="n">
+        <v/>
+      </c>
+      <c r="AR177" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="AS177" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type); Firm Website (family-office status, type)</t>
+        </is>
+      </c>
+      <c r="AT177" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AU177" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AV177" t="inlineStr">
+        <is>
+          <t>corporate_linkedin; principal_linkedin; principal_email; firm_contact_email; principal_name; principal_title; principal_phone; estimated_aum</t>
+        </is>
+      </c>
+      <c r="AW177" t="inlineStr">
+        <is>
+          <t>same-source: discovered via SEC 13F full-text search on filings; verified via the distinct SEC submissions registration record and the firm's regulatory self-identification as a family office</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>fo_9ef7b4677a</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>ELYSEUM FAMILY OFFICE S.A.</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Undetermined</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>SEC Form ADV / IAPD registration names it a family office; firm website describes itself as a family office; type: single vs multi family not established</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Founded in 2011, Elyseum Investment provide first-rate investment services its clients with a focus on Private Equity, Real Estate and Family Office.</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Founded in 2011, Elyseum Investment provides first-rate investment services to its clients with a focus on Private Equity, Real Estate and Family Office.</t>
+        </is>
+      </c>
+      <c r="G178" t="n">
+        <v/>
+      </c>
+      <c r="H178" t="n">
+        <v/>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>https://www.elyseum-investment.com/</t>
+        </is>
+      </c>
+      <c r="J178" t="n">
+        <v/>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>GENEVA</t>
+        </is>
+      </c>
+      <c r="L178" t="n">
+        <v/>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="N178" t="n">
+        <v/>
+      </c>
+      <c r="O178" t="n">
+        <v/>
+      </c>
+      <c r="P178" t="n">
+        <v/>
+      </c>
+      <c r="Q178" t="n">
+        <v/>
+      </c>
+      <c r="R178" t="n">
+        <v/>
+      </c>
+      <c r="S178" t="n">
+        <v/>
+      </c>
+      <c r="T178" t="n">
+        <v/>
+      </c>
+      <c r="U178" t="n">
+        <v/>
+      </c>
+      <c r="V178" t="n">
+        <v/>
+      </c>
+      <c r="W178" t="n">
+        <v/>
+      </c>
+      <c r="X178" t="n">
+        <v/>
+      </c>
+      <c r="Y178" t="n">
+        <v/>
+      </c>
+      <c r="Z178" t="n">
+        <v/>
+      </c>
+      <c r="AA178" t="n">
+        <v/>
+      </c>
+      <c r="AB178" t="n">
+        <v/>
+      </c>
+      <c r="AC178" t="n">
+        <v/>
+      </c>
+      <c r="AD178" t="n">
+        <v/>
+      </c>
+      <c r="AE178" t="n">
+        <v/>
+      </c>
+      <c r="AF178" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AG178" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AH178" t="n">
+        <v/>
+      </c>
+      <c r="AI178" t="n">
+        <v/>
+      </c>
+      <c r="AJ178" t="n">
+        <v/>
+      </c>
+      <c r="AK178" t="n">
+        <v/>
+      </c>
+      <c r="AL178" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AM178" t="n">
+        <v/>
+      </c>
+      <c r="AN178" t="n">
+        <v/>
+      </c>
+      <c r="AO178" t="n">
+        <v/>
+      </c>
+      <c r="AP178" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AQ178" t="n">
+        <v/>
+      </c>
+      <c r="AR178" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="AS178" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type); Firm Website (family-office status, type)</t>
+        </is>
+      </c>
+      <c r="AT178" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AU178" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AV178" t="inlineStr">
+        <is>
+          <t>corporate_linkedin; principal_linkedin; principal_email; firm_contact_email; principal_name; principal_title; principal_phone; estimated_aum</t>
+        </is>
+      </c>
+      <c r="AW178" t="inlineStr">
+        <is>
+          <t>same-source: discovered via SEC 13F full-text search on filings; verified via the distinct SEC submissions registration record and the firm's regulatory self-identification as a family office</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>fo_30c545d0e9</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>ALCALA MULTI FAMILY OFFICE</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Multi-Family Office</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>SEC Form ADV / IAPD registration names it a family office; firm website describes itself as a family office; type: multi-family language</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Ofrecemos asesoría integral y estrategias personalizadas para asegurar el futuro financiero de tu familia.</t>
+        </is>
+      </c>
+      <c r="F179" t="n">
+        <v/>
+      </c>
+      <c r="G179" t="n">
+        <v/>
+      </c>
+      <c r="H179" t="n">
+        <v/>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>https://www.alcala-inversiones.com/es/inicio</t>
+        </is>
+      </c>
+      <c r="J179" t="n">
+        <v/>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>NEW YORK</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="N179" t="n">
+        <v/>
+      </c>
+      <c r="O179" t="n">
+        <v/>
+      </c>
+      <c r="P179" t="n">
+        <v/>
+      </c>
+      <c r="Q179" t="n">
+        <v/>
+      </c>
+      <c r="R179" t="n">
+        <v/>
+      </c>
+      <c r="S179" t="n">
+        <v/>
+      </c>
+      <c r="T179" t="n">
+        <v/>
+      </c>
+      <c r="U179" t="n">
+        <v/>
+      </c>
+      <c r="V179" t="n">
+        <v/>
+      </c>
+      <c r="W179" t="n">
+        <v/>
+      </c>
+      <c r="X179" t="n">
+        <v/>
+      </c>
+      <c r="Y179" t="n">
+        <v/>
+      </c>
+      <c r="Z179" t="n">
+        <v/>
+      </c>
+      <c r="AA179" t="n">
+        <v/>
+      </c>
+      <c r="AB179" t="n">
+        <v/>
+      </c>
+      <c r="AC179" t="n">
+        <v/>
+      </c>
+      <c r="AD179" t="n">
+        <v/>
+      </c>
+      <c r="AE179" t="n">
+        <v/>
+      </c>
+      <c r="AF179" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AG179" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AH179" t="n">
+        <v/>
+      </c>
+      <c r="AI179" t="n">
+        <v/>
+      </c>
+      <c r="AJ179" t="n">
+        <v/>
+      </c>
+      <c r="AK179" t="n">
+        <v/>
+      </c>
+      <c r="AL179" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AM179" t="n">
+        <v/>
+      </c>
+      <c r="AN179" t="n">
+        <v/>
+      </c>
+      <c r="AO179" t="n">
+        <v/>
+      </c>
+      <c r="AP179" t="n">
+        <v/>
+      </c>
+      <c r="AQ179" t="n">
+        <v/>
+      </c>
+      <c r="AR179" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="AS179" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type); Firm Website (family-office status, type)</t>
+        </is>
+      </c>
+      <c r="AT179" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AU179" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AV179" t="inlineStr">
+        <is>
+          <t>corporate_linkedin; principal_linkedin; principal_email; firm_contact_email; principal_name; principal_title; principal_phone; estimated_aum</t>
+        </is>
+      </c>
+      <c r="AW179" t="inlineStr">
+        <is>
+          <t>same-source: discovered via SEC 13F full-text search on filings; verified via the distinct SEC submissions registration record and the firm's regulatory self-identification as a family office</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>fo_79d6c6baca</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>FIFTH AVENUE FAMILY OFFICE</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Undetermined</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>SEC Form ADV / IAPD registration names it a family office; firm website describes itself as a family office; type: single vs multi family not established</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Fifth Avenue Family Office is a team of talented professionals dedicated to serving a select group of entrepreneurial families. We provide family office services that coordinate, manage, and advise across the full-net-worth spectrum. Our goal is to provide our client families with enhanced peace of mind so they can confidently live their lives, love their families and leave their legacies.</t>
+        </is>
+      </c>
+      <c r="F180" t="n">
+        <v/>
+      </c>
+      <c r="G180" t="n">
+        <v/>
+      </c>
+      <c r="H180" t="n">
+        <v/>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>https://fifthavenuefamily.com/</t>
+        </is>
+      </c>
+      <c r="J180" t="n">
+        <v/>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>NAPLES</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="N180" t="n">
+        <v/>
+      </c>
+      <c r="O180" t="n">
+        <v/>
+      </c>
+      <c r="P180" t="n">
+        <v/>
+      </c>
+      <c r="Q180" t="n">
+        <v/>
+      </c>
+      <c r="R180" t="n">
+        <v/>
+      </c>
+      <c r="S180" t="n">
+        <v/>
+      </c>
+      <c r="T180" t="n">
+        <v/>
+      </c>
+      <c r="U180" t="n">
+        <v/>
+      </c>
+      <c r="V180" t="n">
+        <v/>
+      </c>
+      <c r="W180" t="n">
+        <v/>
+      </c>
+      <c r="X180" t="n">
+        <v/>
+      </c>
+      <c r="Y180" t="n">
+        <v/>
+      </c>
+      <c r="Z180" t="n">
+        <v/>
+      </c>
+      <c r="AA180" t="n">
+        <v/>
+      </c>
+      <c r="AB180" t="n">
+        <v/>
+      </c>
+      <c r="AC180" t="n">
+        <v/>
+      </c>
+      <c r="AD180" t="n">
+        <v/>
+      </c>
+      <c r="AE180" t="n">
+        <v/>
+      </c>
+      <c r="AF180" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AG180" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AH180" t="n">
+        <v/>
+      </c>
+      <c r="AI180" t="n">
+        <v/>
+      </c>
+      <c r="AJ180" t="n">
+        <v/>
+      </c>
+      <c r="AK180" t="n">
+        <v/>
+      </c>
+      <c r="AL180" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AM180" t="n">
+        <v/>
+      </c>
+      <c r="AN180" t="n">
+        <v/>
+      </c>
+      <c r="AO180" t="n">
+        <v/>
+      </c>
+      <c r="AP180" t="n">
+        <v/>
+      </c>
+      <c r="AQ180" t="n">
+        <v/>
+      </c>
+      <c r="AR180" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="AS180" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type); Firm Website (family-office status, type)</t>
+        </is>
+      </c>
+      <c r="AT180" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AU180" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AV180" t="inlineStr">
+        <is>
+          <t>corporate_linkedin; principal_linkedin; principal_email; firm_contact_email; principal_name; principal_title; principal_phone; estimated_aum</t>
+        </is>
+      </c>
+      <c r="AW180" t="inlineStr">
+        <is>
+          <t>same-source: discovered via SEC 13F full-text search on filings; verified via the distinct SEC submissions registration record and the firm's regulatory self-identification as a family office</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>fo_cf7e79b88a</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>LEGACY ROAD FAMILY OFFICES</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Undetermined</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>SEC Form ADV / IAPD registration names it a family office; firm website describes itself as a family office; type: single vs multi family not established</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Preserve and grow what matters most. Legacy Road Family Offices delivers expert wealth management and financial planning for high-net-worth families and individuals.</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>The mission of Legacy Road is to provide world-class, institutional quality, investment management and family office services designed to meet the diverse needs of professional athletes, entertainers, and exceptionally affluent individuals and families.</t>
+        </is>
+      </c>
+      <c r="G181" t="n">
+        <v/>
+      </c>
+      <c r="H181" t="n">
+        <v/>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>https://www.legacyroad.com/</t>
+        </is>
+      </c>
+      <c r="J181" t="n">
+        <v/>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="N181" t="n">
+        <v/>
+      </c>
+      <c r="O181" t="n">
+        <v/>
+      </c>
+      <c r="P181" t="n">
+        <v/>
+      </c>
+      <c r="Q181" t="n">
+        <v/>
+      </c>
+      <c r="R181" t="n">
+        <v/>
+      </c>
+      <c r="S181" t="n">
+        <v/>
+      </c>
+      <c r="T181" t="n">
+        <v/>
+      </c>
+      <c r="U181" t="n">
+        <v/>
+      </c>
+      <c r="V181" t="n">
+        <v/>
+      </c>
+      <c r="W181" t="n">
+        <v/>
+      </c>
+      <c r="X181" t="n">
+        <v/>
+      </c>
+      <c r="Y181" t="n">
+        <v/>
+      </c>
+      <c r="Z181" t="n">
+        <v/>
+      </c>
+      <c r="AA181" t="n">
+        <v/>
+      </c>
+      <c r="AB181" t="n">
+        <v/>
+      </c>
+      <c r="AC181" t="n">
+        <v/>
+      </c>
+      <c r="AD181" t="n">
+        <v/>
+      </c>
+      <c r="AE181" t="n">
+        <v/>
+      </c>
+      <c r="AF181" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AG181" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AH181" t="n">
+        <v/>
+      </c>
+      <c r="AI181" t="n">
+        <v/>
+      </c>
+      <c r="AJ181" t="n">
+        <v/>
+      </c>
+      <c r="AK181" t="n">
+        <v/>
+      </c>
+      <c r="AL181" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AM181" t="n">
+        <v/>
+      </c>
+      <c r="AN181" t="n">
+        <v/>
+      </c>
+      <c r="AO181" t="n">
+        <v/>
+      </c>
+      <c r="AP181" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AQ181" t="n">
+        <v/>
+      </c>
+      <c r="AR181" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="AS181" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type); Firm Website (family-office status, type)</t>
+        </is>
+      </c>
+      <c r="AT181" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AU181" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AV181" t="inlineStr">
+        <is>
+          <t>corporate_linkedin; principal_linkedin; principal_email; firm_contact_email; principal_name; principal_title; principal_phone; estimated_aum</t>
+        </is>
+      </c>
+      <c r="AW181" t="inlineStr">
+        <is>
+          <t>same-source: discovered via SEC 13F full-text search on filings; verified via the distinct SEC submissions registration record and the firm's regulatory self-identification as a family office</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>fo_ef3c1aeb59</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>MACI FAMILY OFFICE ADVISORS</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Undetermined</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>SEC Form ADV / IAPD registration names it a family office; firm website describes itself as a family office; type: single vs multi family not established</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Maci capital family office investment advisors new york city</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>We provide comprehensive financial advice, planning, investment &amp; wealth management services to several multi-generational families whose members are spread throughout North America, Europe and Australia.</t>
+        </is>
+      </c>
+      <c r="G182" t="n">
+        <v/>
+      </c>
+      <c r="H182" t="n">
+        <v/>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>https://www.macicapital.com/</t>
+        </is>
+      </c>
+      <c r="J182" t="n">
+        <v/>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>NEW YORK</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="N182" t="n">
+        <v/>
+      </c>
+      <c r="O182" t="n">
+        <v/>
+      </c>
+      <c r="P182" t="n">
+        <v/>
+      </c>
+      <c r="Q182" t="n">
+        <v/>
+      </c>
+      <c r="R182" t="n">
+        <v/>
+      </c>
+      <c r="S182" t="n">
+        <v/>
+      </c>
+      <c r="T182" t="n">
+        <v/>
+      </c>
+      <c r="U182" t="inlineStr">
+        <is>
+          <t>joanne@macicapital.com</t>
+        </is>
+      </c>
+      <c r="V182" t="inlineStr">
+        <is>
+          <t>risky</t>
+        </is>
+      </c>
+      <c r="W182" t="n">
+        <v/>
+      </c>
+      <c r="X182" t="n">
+        <v/>
+      </c>
+      <c r="Y182" t="n">
+        <v/>
+      </c>
+      <c r="Z182" t="n">
+        <v/>
+      </c>
+      <c r="AA182" t="n">
+        <v/>
+      </c>
+      <c r="AB182" t="n">
+        <v/>
+      </c>
+      <c r="AC182" t="n">
+        <v/>
+      </c>
+      <c r="AD182" t="n">
+        <v/>
+      </c>
+      <c r="AE182" t="n">
+        <v/>
+      </c>
+      <c r="AF182" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AG182" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AH182" t="n">
+        <v/>
+      </c>
+      <c r="AI182" t="n">
+        <v/>
+      </c>
+      <c r="AJ182" t="n">
+        <v/>
+      </c>
+      <c r="AK182" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AL182" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AM182" t="n">
+        <v/>
+      </c>
+      <c r="AN182" t="n">
+        <v/>
+      </c>
+      <c r="AO182" t="n">
+        <v/>
+      </c>
+      <c r="AP182" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AQ182" t="n">
+        <v/>
+      </c>
+      <c r="AR182" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="AS182" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type); Firm Website (family-office status, type)</t>
+        </is>
+      </c>
+      <c r="AT182" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AU182" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AV182" t="inlineStr">
+        <is>
+          <t>corporate_linkedin; principal_linkedin; principal_email; principal_name; principal_title; principal_phone; estimated_aum</t>
+        </is>
+      </c>
+      <c r="AW182" t="inlineStr">
+        <is>
+          <t>same-source: discovered via SEC 13F full-text search on filings; verified via the distinct SEC submissions registration record and the firm's regulatory self-identification as a family office | firm_contact_email is the firm's published contact inbox (official site) — a real, sourced channel but not a route to any named individual</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>fo_1ed11ef389</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>QP GLOBAL FAMILY OFFICES, LLC</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Single-Family Office</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>SEC Form ADV / IAPD registration names it a family office; firm website describes itself as a family office; type: single-family language</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Elite single-family office management: Full ownership and control for discerning families. We handle design, leadership, staffing, operations, investments, and governance—so you focus on legacy and life.</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Our shared model means: You own everything — your wealth, your vision, your decisions, your legacy.</t>
+        </is>
+      </c>
+      <c r="G183" t="n">
+        <v/>
+      </c>
+      <c r="H183" t="n">
+        <v/>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>https://www.qp-global.com/</t>
+        </is>
+      </c>
+      <c r="J183" t="n">
+        <v/>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>GREENWICH</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="N183" t="n">
+        <v/>
+      </c>
+      <c r="O183" t="n">
+        <v/>
+      </c>
+      <c r="P183" t="n">
+        <v/>
+      </c>
+      <c r="Q183" t="n">
+        <v/>
+      </c>
+      <c r="R183" t="n">
+        <v/>
+      </c>
+      <c r="S183" t="n">
+        <v/>
+      </c>
+      <c r="T183" t="n">
+        <v/>
+      </c>
+      <c r="U183" t="inlineStr">
+        <is>
+          <t>info@qp-global.com</t>
+        </is>
+      </c>
+      <c r="V183" t="inlineStr">
+        <is>
+          <t>risky</t>
+        </is>
+      </c>
+      <c r="W183" t="n">
+        <v/>
+      </c>
+      <c r="X183" t="n">
+        <v/>
+      </c>
+      <c r="Y183" t="n">
+        <v/>
+      </c>
+      <c r="Z183" t="n">
+        <v/>
+      </c>
+      <c r="AA183" t="n">
+        <v/>
+      </c>
+      <c r="AB183" t="n">
+        <v/>
+      </c>
+      <c r="AC183" t="n">
+        <v/>
+      </c>
+      <c r="AD183" t="n">
+        <v/>
+      </c>
+      <c r="AE183" t="n">
+        <v/>
+      </c>
+      <c r="AF183" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AG183" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AH183" t="n">
+        <v/>
+      </c>
+      <c r="AI183" t="n">
+        <v/>
+      </c>
+      <c r="AJ183" t="n">
+        <v/>
+      </c>
+      <c r="AK183" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AL183" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AM183" t="n">
+        <v/>
+      </c>
+      <c r="AN183" t="n">
+        <v/>
+      </c>
+      <c r="AO183" t="n">
+        <v/>
+      </c>
+      <c r="AP183" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AQ183" t="n">
+        <v/>
+      </c>
+      <c r="AR183" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration)</t>
+        </is>
+      </c>
+      <c r="AS183" t="inlineStr">
+        <is>
+          <t>SEC IAPD / Form ADV (investment-adviser registration) (firm registration, family-office status, type); Firm Website (family-office status, type)</t>
+        </is>
+      </c>
+      <c r="AT183" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AU183" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AV183" t="inlineStr">
+        <is>
+          <t>corporate_linkedin; principal_linkedin; principal_email; principal_name; principal_title; principal_phone; estimated_aum</t>
+        </is>
+      </c>
+      <c r="AW183" t="inlineStr">
+        <is>
+          <t>same-source: discovered via SEC 13F full-text search on filings; verified via the distinct SEC submissions registration record and the firm's regulatory self-identification as a family office | firm_contact_email is the firm's published contact inbox (official site) — a real, sourced channel but not a route to any named individual</t>
         </is>
       </c>
     </row>

</xml_diff>